<commit_message>
extra logging and added Peer to data
</commit_message>
<xml_diff>
--- a/Excel_files/Log/Grocery_List_Log.xlsx
+++ b/Excel_files/Log/Grocery_List_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elskn\Projects\Grocery_list\Excel_files\Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70AD4F92-AF9F-4DB7-B5EC-4AAF7C4D841A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0623E994-E7F6-4F6C-B539-D043D2CAAB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Log Per Recipe" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3564" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3886" uniqueCount="188">
   <si>
     <t>Recipe</t>
   </si>
@@ -658,7 +658,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -666,8 +666,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -1409,7 +1407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G588"/>
+  <dimension ref="A1:G642"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="29.26171875" bestFit="1" customWidth="1"/>
@@ -13952,22 +13950,22 @@
       </c>
     </row>
     <row r="546" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A546" s="6" t="s">
+      <c r="A546" t="s">
         <v>34</v>
       </c>
-      <c r="B546" s="6">
+      <c r="B546">
         <v>4</v>
       </c>
-      <c r="C546" s="6" t="s">
+      <c r="C546" t="s">
         <v>16</v>
       </c>
-      <c r="D546" s="6" t="s">
+      <c r="D546" t="s">
         <v>17</v>
       </c>
-      <c r="E546" s="6">
+      <c r="E546">
         <v>240</v>
       </c>
-      <c r="F546" s="6" t="s">
+      <c r="F546" t="s">
         <v>10</v>
       </c>
       <c r="G546" s="2">
@@ -13975,22 +13973,22 @@
       </c>
     </row>
     <row r="547" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A547" s="6" t="s">
+      <c r="A547" t="s">
         <v>34</v>
       </c>
-      <c r="B547" s="6">
+      <c r="B547">
         <v>4</v>
       </c>
-      <c r="C547" s="6" t="s">
+      <c r="C547" t="s">
         <v>35</v>
       </c>
-      <c r="D547" s="6" t="s">
+      <c r="D547" t="s">
         <v>36</v>
       </c>
-      <c r="E547" s="6">
+      <c r="E547">
         <v>256</v>
       </c>
-      <c r="F547" s="6" t="s">
+      <c r="F547" t="s">
         <v>10</v>
       </c>
       <c r="G547" s="2">
@@ -13998,22 +13996,22 @@
       </c>
     </row>
     <row r="548" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A548" s="6" t="s">
+      <c r="A548" t="s">
         <v>34</v>
       </c>
-      <c r="B548" s="6">
+      <c r="B548">
         <v>4</v>
       </c>
-      <c r="C548" s="6" t="s">
+      <c r="C548" t="s">
         <v>37</v>
       </c>
-      <c r="D548" s="6" t="s">
+      <c r="D548" t="s">
         <v>38</v>
       </c>
-      <c r="E548" s="6">
+      <c r="E548">
         <v>1</v>
       </c>
-      <c r="F548" s="6" t="s">
+      <c r="F548" t="s">
         <v>15</v>
       </c>
       <c r="G548" s="2">
@@ -14021,22 +14019,22 @@
       </c>
     </row>
     <row r="549" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A549" s="6" t="s">
+      <c r="A549" t="s">
         <v>34</v>
       </c>
-      <c r="B549" s="6">
+      <c r="B549">
         <v>4</v>
       </c>
-      <c r="C549" s="6" t="s">
+      <c r="C549" t="s">
         <v>39</v>
       </c>
-      <c r="D549" s="6" t="s">
+      <c r="D549" t="s">
         <v>40</v>
       </c>
-      <c r="E549" s="6">
+      <c r="E549">
         <v>0.68</v>
       </c>
-      <c r="F549" s="6" t="s">
+      <c r="F549" t="s">
         <v>15</v>
       </c>
       <c r="G549" s="2">
@@ -14044,22 +14042,22 @@
       </c>
     </row>
     <row r="550" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A550" s="6" t="s">
+      <c r="A550" t="s">
         <v>34</v>
       </c>
-      <c r="B550" s="6">
+      <c r="B550">
         <v>4</v>
       </c>
-      <c r="C550" s="6" t="s">
+      <c r="C550" t="s">
         <v>24</v>
       </c>
-      <c r="D550" s="6" t="s">
+      <c r="D550" t="s">
         <v>25</v>
       </c>
-      <c r="E550" s="6">
+      <c r="E550">
         <v>1</v>
       </c>
-      <c r="F550" s="6" t="s">
+      <c r="F550" t="s">
         <v>15</v>
       </c>
       <c r="G550" s="2">
@@ -14067,22 +14065,22 @@
       </c>
     </row>
     <row r="551" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A551" s="6" t="s">
+      <c r="A551" t="s">
         <v>34</v>
       </c>
-      <c r="B551" s="6">
+      <c r="B551">
         <v>4</v>
       </c>
-      <c r="C551" s="6" t="s">
+      <c r="C551" t="s">
         <v>41</v>
       </c>
-      <c r="D551" s="6" t="s">
+      <c r="D551" t="s">
         <v>42</v>
       </c>
-      <c r="E551" s="6">
+      <c r="E551">
         <v>2</v>
       </c>
-      <c r="F551" s="6" t="s">
+      <c r="F551" t="s">
         <v>15</v>
       </c>
       <c r="G551" s="2">
@@ -14090,22 +14088,22 @@
       </c>
     </row>
     <row r="552" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A552" s="6" t="s">
+      <c r="A552" t="s">
         <v>34</v>
       </c>
-      <c r="B552" s="6">
+      <c r="B552">
         <v>4</v>
       </c>
-      <c r="C552" s="6" t="s">
+      <c r="C552" t="s">
         <v>43</v>
       </c>
-      <c r="D552" s="6" t="s">
+      <c r="D552" t="s">
         <v>44</v>
       </c>
-      <c r="E552" s="6">
+      <c r="E552">
         <v>200</v>
       </c>
-      <c r="F552" s="6" t="s">
+      <c r="F552" t="s">
         <v>10</v>
       </c>
       <c r="G552" s="2">
@@ -14113,22 +14111,22 @@
       </c>
     </row>
     <row r="553" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A553" s="6" t="s">
+      <c r="A553" t="s">
         <v>34</v>
       </c>
-      <c r="B553" s="6">
+      <c r="B553">
         <v>4</v>
       </c>
-      <c r="C553" s="6" t="s">
+      <c r="C553" t="s">
         <v>45</v>
       </c>
-      <c r="D553" s="6" t="s">
+      <c r="D553" t="s">
         <v>46</v>
       </c>
-      <c r="E553" s="6">
+      <c r="E553">
         <v>40</v>
       </c>
-      <c r="F553" s="6" t="s">
+      <c r="F553" t="s">
         <v>10</v>
       </c>
       <c r="G553" s="2">
@@ -14136,22 +14134,22 @@
       </c>
     </row>
     <row r="554" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A554" s="6" t="s">
+      <c r="A554" t="s">
         <v>34</v>
       </c>
-      <c r="B554" s="6">
+      <c r="B554">
         <v>4</v>
       </c>
-      <c r="C554" s="6" t="s">
+      <c r="C554" t="s">
         <v>47</v>
       </c>
-      <c r="D554" s="6" t="s">
+      <c r="D554" t="s">
         <v>48</v>
       </c>
-      <c r="E554" s="6">
+      <c r="E554">
         <v>50</v>
       </c>
-      <c r="F554" s="6" t="s">
+      <c r="F554" t="s">
         <v>10</v>
       </c>
       <c r="G554" s="2">
@@ -14159,22 +14157,22 @@
       </c>
     </row>
     <row r="555" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A555" s="6" t="s">
+      <c r="A555" t="s">
         <v>34</v>
       </c>
-      <c r="B555" s="6">
+      <c r="B555">
         <v>4</v>
       </c>
-      <c r="C555" s="6" t="s">
+      <c r="C555" t="s">
         <v>20</v>
       </c>
-      <c r="D555" s="6" t="s">
+      <c r="D555" t="s">
         <v>21</v>
       </c>
-      <c r="E555" s="6">
+      <c r="E555">
         <v>50</v>
       </c>
-      <c r="F555" s="6" t="s">
+      <c r="F555" t="s">
         <v>10</v>
       </c>
       <c r="G555" s="2">
@@ -14182,22 +14180,22 @@
       </c>
     </row>
     <row r="556" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A556" s="6" t="s">
+      <c r="A556" t="s">
         <v>34</v>
       </c>
-      <c r="B556" s="6">
+      <c r="B556">
         <v>4</v>
       </c>
-      <c r="C556" s="6" t="s">
+      <c r="C556" t="s">
         <v>53</v>
       </c>
-      <c r="D556" s="6" t="s">
+      <c r="D556" t="s">
         <v>54</v>
       </c>
-      <c r="E556" s="6">
+      <c r="E556">
         <v>8</v>
       </c>
-      <c r="F556" s="6" t="s">
+      <c r="F556" t="s">
         <v>15</v>
       </c>
       <c r="G556" s="2">
@@ -14205,22 +14203,22 @@
       </c>
     </row>
     <row r="557" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A557" s="6" t="s">
+      <c r="A557" t="s">
         <v>34</v>
       </c>
-      <c r="B557" s="6">
+      <c r="B557">
         <v>4</v>
       </c>
-      <c r="C557" s="6" t="s">
+      <c r="C557" t="s">
         <v>55</v>
       </c>
-      <c r="D557" s="6" t="s">
+      <c r="D557" t="s">
         <v>56</v>
       </c>
-      <c r="E557" s="6">
+      <c r="E557">
         <v>120</v>
       </c>
-      <c r="F557" s="6" t="s">
+      <c r="F557" t="s">
         <v>10</v>
       </c>
       <c r="G557" s="2">
@@ -14228,22 +14226,22 @@
       </c>
     </row>
     <row r="558" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A558" s="6" t="s">
+      <c r="A558" t="s">
         <v>130</v>
       </c>
-      <c r="B558" s="6">
+      <c r="B558">
         <v>2</v>
       </c>
-      <c r="C558" s="6" t="s">
+      <c r="C558" t="s">
         <v>35</v>
       </c>
-      <c r="D558" s="6" t="s">
+      <c r="D558" t="s">
         <v>36</v>
       </c>
-      <c r="E558" s="6">
+      <c r="E558">
         <v>128</v>
       </c>
-      <c r="F558" s="6" t="s">
+      <c r="F558" t="s">
         <v>10</v>
       </c>
       <c r="G558" s="2">
@@ -14251,22 +14249,22 @@
       </c>
     </row>
     <row r="559" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A559" s="6" t="s">
+      <c r="A559" t="s">
         <v>130</v>
       </c>
-      <c r="B559" s="6">
+      <c r="B559">
         <v>2</v>
       </c>
-      <c r="C559" s="6" t="s">
+      <c r="C559" t="s">
         <v>37</v>
       </c>
-      <c r="D559" s="6" t="s">
+      <c r="D559" t="s">
         <v>38</v>
       </c>
-      <c r="E559" s="6">
+      <c r="E559">
         <v>0.5</v>
       </c>
-      <c r="F559" s="6" t="s">
+      <c r="F559" t="s">
         <v>15</v>
       </c>
       <c r="G559" s="2">
@@ -14274,22 +14272,22 @@
       </c>
     </row>
     <row r="560" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A560" s="6" t="s">
+      <c r="A560" t="s">
         <v>130</v>
       </c>
-      <c r="B560" s="6">
+      <c r="B560">
         <v>2</v>
       </c>
-      <c r="C560" s="6" t="s">
+      <c r="C560" t="s">
         <v>39</v>
       </c>
-      <c r="D560" s="6" t="s">
+      <c r="D560" t="s">
         <v>40</v>
       </c>
-      <c r="E560" s="6">
+      <c r="E560">
         <v>0.34</v>
       </c>
-      <c r="F560" s="6" t="s">
+      <c r="F560" t="s">
         <v>15</v>
       </c>
       <c r="G560" s="2">
@@ -14297,22 +14295,22 @@
       </c>
     </row>
     <row r="561" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A561" s="6" t="s">
+      <c r="A561" t="s">
         <v>130</v>
       </c>
-      <c r="B561" s="6">
+      <c r="B561">
         <v>2</v>
       </c>
-      <c r="C561" s="6" t="s">
+      <c r="C561" t="s">
         <v>24</v>
       </c>
-      <c r="D561" s="6" t="s">
+      <c r="D561" t="s">
         <v>25</v>
       </c>
-      <c r="E561" s="6">
+      <c r="E561">
         <v>0.5</v>
       </c>
-      <c r="F561" s="6" t="s">
+      <c r="F561" t="s">
         <v>15</v>
       </c>
       <c r="G561" s="2">
@@ -14320,22 +14318,22 @@
       </c>
     </row>
     <row r="562" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A562" s="6" t="s">
+      <c r="A562" t="s">
         <v>130</v>
       </c>
-      <c r="B562" s="6">
+      <c r="B562">
         <v>2</v>
       </c>
-      <c r="C562" s="6" t="s">
+      <c r="C562" t="s">
         <v>41</v>
       </c>
-      <c r="D562" s="6" t="s">
+      <c r="D562" t="s">
         <v>42</v>
       </c>
-      <c r="E562" s="6">
+      <c r="E562">
         <v>1</v>
       </c>
-      <c r="F562" s="6" t="s">
+      <c r="F562" t="s">
         <v>15</v>
       </c>
       <c r="G562" s="2">
@@ -14343,22 +14341,22 @@
       </c>
     </row>
     <row r="563" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A563" s="6" t="s">
+      <c r="A563" t="s">
         <v>130</v>
       </c>
-      <c r="B563" s="6">
+      <c r="B563">
         <v>2</v>
       </c>
-      <c r="C563" s="6" t="s">
+      <c r="C563" t="s">
         <v>43</v>
       </c>
-      <c r="D563" s="6" t="s">
+      <c r="D563" t="s">
         <v>44</v>
       </c>
-      <c r="E563" s="6">
+      <c r="E563">
         <v>100</v>
       </c>
-      <c r="F563" s="6" t="s">
+      <c r="F563" t="s">
         <v>10</v>
       </c>
       <c r="G563" s="2">
@@ -14366,22 +14364,22 @@
       </c>
     </row>
     <row r="564" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A564" s="6" t="s">
+      <c r="A564" t="s">
         <v>130</v>
       </c>
-      <c r="B564" s="6">
+      <c r="B564">
         <v>2</v>
       </c>
-      <c r="C564" s="6" t="s">
+      <c r="C564" t="s">
         <v>45</v>
       </c>
-      <c r="D564" s="6" t="s">
+      <c r="D564" t="s">
         <v>46</v>
       </c>
-      <c r="E564" s="6">
+      <c r="E564">
         <v>20</v>
       </c>
-      <c r="F564" s="6" t="s">
+      <c r="F564" t="s">
         <v>10</v>
       </c>
       <c r="G564" s="2">
@@ -14389,22 +14387,22 @@
       </c>
     </row>
     <row r="565" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A565" s="6" t="s">
+      <c r="A565" t="s">
         <v>130</v>
       </c>
-      <c r="B565" s="6">
+      <c r="B565">
         <v>2</v>
       </c>
-      <c r="C565" s="6" t="s">
+      <c r="C565" t="s">
         <v>47</v>
       </c>
-      <c r="D565" s="6" t="s">
+      <c r="D565" t="s">
         <v>48</v>
       </c>
-      <c r="E565" s="6">
+      <c r="E565">
         <v>25</v>
       </c>
-      <c r="F565" s="6" t="s">
+      <c r="F565" t="s">
         <v>10</v>
       </c>
       <c r="G565" s="2">
@@ -14412,22 +14410,22 @@
       </c>
     </row>
     <row r="566" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A566" s="6" t="s">
+      <c r="A566" t="s">
         <v>130</v>
       </c>
-      <c r="B566" s="6">
+      <c r="B566">
         <v>2</v>
       </c>
-      <c r="C566" s="6" t="s">
+      <c r="C566" t="s">
         <v>16</v>
       </c>
-      <c r="D566" s="6" t="s">
+      <c r="D566" t="s">
         <v>17</v>
       </c>
-      <c r="E566" s="6">
+      <c r="E566">
         <v>120</v>
       </c>
-      <c r="F566" s="6" t="s">
+      <c r="F566" t="s">
         <v>10</v>
       </c>
       <c r="G566" s="2">
@@ -14435,22 +14433,22 @@
       </c>
     </row>
     <row r="567" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A567" s="6" t="s">
+      <c r="A567" t="s">
         <v>130</v>
       </c>
-      <c r="B567" s="6">
+      <c r="B567">
         <v>2</v>
       </c>
-      <c r="C567" s="6" t="s">
+      <c r="C567" t="s">
         <v>20</v>
       </c>
-      <c r="D567" s="6" t="s">
+      <c r="D567" t="s">
         <v>21</v>
       </c>
-      <c r="E567" s="6">
+      <c r="E567">
         <v>25</v>
       </c>
-      <c r="F567" s="6" t="s">
+      <c r="F567" t="s">
         <v>10</v>
       </c>
       <c r="G567" s="2">
@@ -14458,22 +14456,22 @@
       </c>
     </row>
     <row r="568" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A568" s="6" t="s">
+      <c r="A568" t="s">
         <v>131</v>
       </c>
-      <c r="B568" s="6">
+      <c r="B568">
         <v>6</v>
       </c>
-      <c r="C568" s="6" t="s">
+      <c r="C568" t="s">
         <v>35</v>
       </c>
-      <c r="D568" s="6" t="s">
+      <c r="D568" t="s">
         <v>36</v>
       </c>
-      <c r="E568" s="6">
+      <c r="E568">
         <v>384</v>
       </c>
-      <c r="F568" s="6" t="s">
+      <c r="F568" t="s">
         <v>10</v>
       </c>
       <c r="G568" s="2">
@@ -14481,22 +14479,22 @@
       </c>
     </row>
     <row r="569" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A569" s="6" t="s">
+      <c r="A569" t="s">
         <v>131</v>
       </c>
-      <c r="B569" s="6">
+      <c r="B569">
         <v>6</v>
       </c>
-      <c r="C569" s="6" t="s">
+      <c r="C569" t="s">
         <v>37</v>
       </c>
-      <c r="D569" s="6" t="s">
+      <c r="D569" t="s">
         <v>38</v>
       </c>
-      <c r="E569" s="6">
+      <c r="E569">
         <v>1.5</v>
       </c>
-      <c r="F569" s="6" t="s">
+      <c r="F569" t="s">
         <v>15</v>
       </c>
       <c r="G569" s="2">
@@ -14504,22 +14502,22 @@
       </c>
     </row>
     <row r="570" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A570" s="6" t="s">
+      <c r="A570" t="s">
         <v>131</v>
       </c>
-      <c r="B570" s="6">
+      <c r="B570">
         <v>6</v>
       </c>
-      <c r="C570" s="6" t="s">
+      <c r="C570" t="s">
         <v>39</v>
       </c>
-      <c r="D570" s="6" t="s">
+      <c r="D570" t="s">
         <v>40</v>
       </c>
-      <c r="E570" s="6">
+      <c r="E570">
         <v>1.02</v>
       </c>
-      <c r="F570" s="6" t="s">
+      <c r="F570" t="s">
         <v>15</v>
       </c>
       <c r="G570" s="2">
@@ -14527,22 +14525,22 @@
       </c>
     </row>
     <row r="571" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A571" s="6" t="s">
+      <c r="A571" t="s">
         <v>131</v>
       </c>
-      <c r="B571" s="6">
+      <c r="B571">
         <v>6</v>
       </c>
-      <c r="C571" s="6" t="s">
+      <c r="C571" t="s">
         <v>24</v>
       </c>
-      <c r="D571" s="6" t="s">
+      <c r="D571" t="s">
         <v>25</v>
       </c>
-      <c r="E571" s="6">
+      <c r="E571">
         <v>1.5</v>
       </c>
-      <c r="F571" s="6" t="s">
+      <c r="F571" t="s">
         <v>15</v>
       </c>
       <c r="G571" s="2">
@@ -14550,22 +14548,22 @@
       </c>
     </row>
     <row r="572" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A572" s="6" t="s">
+      <c r="A572" t="s">
         <v>131</v>
       </c>
-      <c r="B572" s="6">
+      <c r="B572">
         <v>6</v>
       </c>
-      <c r="C572" s="6" t="s">
+      <c r="C572" t="s">
         <v>41</v>
       </c>
-      <c r="D572" s="6" t="s">
+      <c r="D572" t="s">
         <v>42</v>
       </c>
-      <c r="E572" s="6">
+      <c r="E572">
         <v>3</v>
       </c>
-      <c r="F572" s="6" t="s">
+      <c r="F572" t="s">
         <v>15</v>
       </c>
       <c r="G572" s="2">
@@ -14573,22 +14571,22 @@
       </c>
     </row>
     <row r="573" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A573" s="6" t="s">
+      <c r="A573" t="s">
         <v>131</v>
       </c>
-      <c r="B573" s="6">
+      <c r="B573">
         <v>6</v>
       </c>
-      <c r="C573" s="6" t="s">
+      <c r="C573" t="s">
         <v>43</v>
       </c>
-      <c r="D573" s="6" t="s">
+      <c r="D573" t="s">
         <v>44</v>
       </c>
-      <c r="E573" s="6">
+      <c r="E573">
         <v>300</v>
       </c>
-      <c r="F573" s="6" t="s">
+      <c r="F573" t="s">
         <v>10</v>
       </c>
       <c r="G573" s="2">
@@ -14596,22 +14594,22 @@
       </c>
     </row>
     <row r="574" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A574" s="6" t="s">
+      <c r="A574" t="s">
         <v>131</v>
       </c>
-      <c r="B574" s="6">
+      <c r="B574">
         <v>6</v>
       </c>
-      <c r="C574" s="6" t="s">
+      <c r="C574" t="s">
         <v>45</v>
       </c>
-      <c r="D574" s="6" t="s">
+      <c r="D574" t="s">
         <v>46</v>
       </c>
-      <c r="E574" s="6">
+      <c r="E574">
         <v>60</v>
       </c>
-      <c r="F574" s="6" t="s">
+      <c r="F574" t="s">
         <v>10</v>
       </c>
       <c r="G574" s="2">
@@ -14619,22 +14617,22 @@
       </c>
     </row>
     <row r="575" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A575" s="6" t="s">
+      <c r="A575" t="s">
         <v>131</v>
       </c>
-      <c r="B575" s="6">
+      <c r="B575">
         <v>6</v>
       </c>
-      <c r="C575" s="6" t="s">
+      <c r="C575" t="s">
         <v>47</v>
       </c>
-      <c r="D575" s="6" t="s">
+      <c r="D575" t="s">
         <v>48</v>
       </c>
-      <c r="E575" s="6">
+      <c r="E575">
         <v>75</v>
       </c>
-      <c r="F575" s="6" t="s">
+      <c r="F575" t="s">
         <v>10</v>
       </c>
       <c r="G575" s="2">
@@ -14642,22 +14640,22 @@
       </c>
     </row>
     <row r="576" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A576" s="6" t="s">
+      <c r="A576" t="s">
         <v>131</v>
       </c>
-      <c r="B576" s="6">
+      <c r="B576">
         <v>6</v>
       </c>
-      <c r="C576" s="6" t="s">
+      <c r="C576" t="s">
         <v>20</v>
       </c>
-      <c r="D576" s="6" t="s">
+      <c r="D576" t="s">
         <v>21</v>
       </c>
-      <c r="E576" s="6">
+      <c r="E576">
         <v>75</v>
       </c>
-      <c r="F576" s="6" t="s">
+      <c r="F576" t="s">
         <v>10</v>
       </c>
       <c r="G576" s="2">
@@ -14665,22 +14663,22 @@
       </c>
     </row>
     <row r="577" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A577" s="6" t="s">
+      <c r="A577" t="s">
         <v>131</v>
       </c>
-      <c r="B577" s="6">
+      <c r="B577">
         <v>6</v>
       </c>
-      <c r="C577" s="6" t="s">
+      <c r="C577" t="s">
         <v>16</v>
       </c>
-      <c r="D577" s="6" t="s">
+      <c r="D577" t="s">
         <v>17</v>
       </c>
-      <c r="E577" s="6">
+      <c r="E577">
         <v>360</v>
       </c>
-      <c r="F577" s="6" t="s">
+      <c r="F577" t="s">
         <v>10</v>
       </c>
       <c r="G577" s="2">
@@ -14688,22 +14686,22 @@
       </c>
     </row>
     <row r="578" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A578" s="6" t="s">
+      <c r="A578" t="s">
         <v>131</v>
       </c>
-      <c r="B578" s="6">
+      <c r="B578">
         <v>6</v>
       </c>
-      <c r="C578" s="6" t="s">
+      <c r="C578" t="s">
         <v>8</v>
       </c>
-      <c r="D578" s="6" t="s">
+      <c r="D578" t="s">
         <v>9</v>
       </c>
-      <c r="E578" s="6">
+      <c r="E578">
         <v>600</v>
       </c>
-      <c r="F578" s="6" t="s">
+      <c r="F578" t="s">
         <v>10</v>
       </c>
       <c r="G578" s="2">
@@ -14711,22 +14709,22 @@
       </c>
     </row>
     <row r="579" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A579" s="6" t="s">
+      <c r="A579" t="s">
         <v>89</v>
       </c>
-      <c r="B579" s="6">
+      <c r="B579">
         <v>6</v>
       </c>
-      <c r="C579" s="6" t="s">
+      <c r="C579" t="s">
         <v>90</v>
       </c>
-      <c r="D579" s="6" t="s">
+      <c r="D579" t="s">
         <v>91</v>
       </c>
-      <c r="E579" s="6">
+      <c r="E579">
         <v>600</v>
       </c>
-      <c r="F579" s="6" t="s">
+      <c r="F579" t="s">
         <v>10</v>
       </c>
       <c r="G579" s="2">
@@ -14734,22 +14732,22 @@
       </c>
     </row>
     <row r="580" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A580" s="6" t="s">
+      <c r="A580" t="s">
         <v>89</v>
       </c>
-      <c r="B580" s="6">
+      <c r="B580">
         <v>6</v>
       </c>
-      <c r="C580" s="6" t="s">
+      <c r="C580" t="s">
         <v>92</v>
       </c>
-      <c r="D580" s="6" t="s">
+      <c r="D580" t="s">
         <v>93</v>
       </c>
-      <c r="E580" s="6">
+      <c r="E580">
         <v>960</v>
       </c>
-      <c r="F580" s="6" t="s">
+      <c r="F580" t="s">
         <v>10</v>
       </c>
       <c r="G580" s="2">
@@ -14757,22 +14755,22 @@
       </c>
     </row>
     <row r="581" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A581" s="6" t="s">
+      <c r="A581" t="s">
         <v>89</v>
       </c>
-      <c r="B581" s="6">
+      <c r="B581">
         <v>6</v>
       </c>
-      <c r="C581" s="6" t="s">
+      <c r="C581" t="s">
         <v>64</v>
       </c>
-      <c r="D581" s="6" t="s">
+      <c r="D581" t="s">
         <v>65</v>
       </c>
-      <c r="E581" s="6">
+      <c r="E581">
         <v>300</v>
       </c>
-      <c r="F581" s="6" t="s">
+      <c r="F581" t="s">
         <v>10</v>
       </c>
       <c r="G581" s="2">
@@ -14780,22 +14778,22 @@
       </c>
     </row>
     <row r="582" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A582" s="6" t="s">
+      <c r="A582" t="s">
         <v>89</v>
       </c>
-      <c r="B582" s="6">
+      <c r="B582">
         <v>6</v>
       </c>
-      <c r="C582" s="6" t="s">
+      <c r="C582" t="s">
         <v>68</v>
       </c>
-      <c r="D582" s="6" t="s">
+      <c r="D582" t="s">
         <v>69</v>
       </c>
-      <c r="E582" s="6">
+      <c r="E582">
         <v>270</v>
       </c>
-      <c r="F582" s="6" t="s">
+      <c r="F582" t="s">
         <v>10</v>
       </c>
       <c r="G582" s="2">
@@ -14803,22 +14801,22 @@
       </c>
     </row>
     <row r="583" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A583" s="6" t="s">
+      <c r="A583" t="s">
         <v>71</v>
       </c>
-      <c r="B583" s="6">
+      <c r="B583">
         <v>4</v>
       </c>
-      <c r="C583" s="6" t="s">
+      <c r="C583" t="s">
         <v>72</v>
       </c>
-      <c r="D583" s="6" t="s">
+      <c r="D583" t="s">
         <v>73</v>
       </c>
-      <c r="E583" s="6">
+      <c r="E583">
         <v>1000</v>
       </c>
-      <c r="F583" s="6" t="s">
+      <c r="F583" t="s">
         <v>10</v>
       </c>
       <c r="G583" s="2">
@@ -14826,22 +14824,22 @@
       </c>
     </row>
     <row r="584" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A584" s="6" t="s">
+      <c r="A584" t="s">
         <v>71</v>
       </c>
-      <c r="B584" s="6">
+      <c r="B584">
         <v>4</v>
       </c>
-      <c r="C584" s="6" t="s">
+      <c r="C584" t="s">
         <v>28</v>
       </c>
-      <c r="D584" s="6" t="s">
+      <c r="D584" t="s">
         <v>29</v>
       </c>
-      <c r="E584" s="6">
+      <c r="E584">
         <v>400</v>
       </c>
-      <c r="F584" s="6" t="s">
+      <c r="F584" t="s">
         <v>10</v>
       </c>
       <c r="G584" s="2">
@@ -14849,22 +14847,22 @@
       </c>
     </row>
     <row r="585" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A585" s="6" t="s">
+      <c r="A585" t="s">
         <v>71</v>
       </c>
-      <c r="B585" s="6">
+      <c r="B585">
         <v>4</v>
       </c>
-      <c r="C585" s="6" t="s">
+      <c r="C585" t="s">
         <v>74</v>
       </c>
-      <c r="D585" s="6" t="s">
+      <c r="D585" t="s">
         <v>75</v>
       </c>
-      <c r="E585" s="6">
+      <c r="E585">
         <v>400</v>
       </c>
-      <c r="F585" s="6" t="s">
+      <c r="F585" t="s">
         <v>10</v>
       </c>
       <c r="G585" s="2">
@@ -14872,22 +14870,22 @@
       </c>
     </row>
     <row r="586" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A586" s="6" t="s">
+      <c r="A586" t="s">
         <v>71</v>
       </c>
-      <c r="B586" s="6">
+      <c r="B586">
         <v>4</v>
       </c>
-      <c r="C586" s="6" t="s">
+      <c r="C586" t="s">
         <v>76</v>
       </c>
-      <c r="D586" s="6" t="s">
+      <c r="D586" t="s">
         <v>77</v>
       </c>
-      <c r="E586" s="6">
+      <c r="E586">
         <v>200</v>
       </c>
-      <c r="F586" s="6" t="s">
+      <c r="F586" t="s">
         <v>10</v>
       </c>
       <c r="G586" s="2">
@@ -14895,22 +14893,22 @@
       </c>
     </row>
     <row r="587" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A587" s="6" t="s">
+      <c r="A587" t="s">
         <v>71</v>
       </c>
-      <c r="B587" s="6">
+      <c r="B587">
         <v>4</v>
       </c>
-      <c r="C587" s="6" t="s">
+      <c r="C587" t="s">
         <v>18</v>
       </c>
-      <c r="D587" s="6" t="s">
+      <c r="D587" t="s">
         <v>19</v>
       </c>
-      <c r="E587" s="6">
+      <c r="E587">
         <v>16</v>
       </c>
-      <c r="F587" s="6" t="s">
+      <c r="F587" t="s">
         <v>15</v>
       </c>
       <c r="G587" s="2">
@@ -14918,27 +14916,1029 @@
       </c>
     </row>
     <row r="588" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A588" s="6" t="s">
+      <c r="A588" t="s">
         <v>71</v>
       </c>
-      <c r="B588" s="6">
+      <c r="B588">
         <v>4</v>
       </c>
-      <c r="C588" s="6" t="s">
+      <c r="C588" t="s">
         <v>78</v>
       </c>
-      <c r="D588" s="6" t="s">
+      <c r="D588" t="s">
         <v>79</v>
       </c>
-      <c r="E588" s="6">
+      <c r="E588">
         <v>8</v>
       </c>
-      <c r="F588" s="6" t="s">
+      <c r="F588" t="s">
         <v>10</v>
       </c>
       <c r="G588" s="2">
         <v>45918</v>
       </c>
+    </row>
+    <row r="589" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A589" t="s">
+        <v>89</v>
+      </c>
+      <c r="B589">
+        <v>6</v>
+      </c>
+      <c r="C589" t="s">
+        <v>90</v>
+      </c>
+      <c r="D589" t="s">
+        <v>91</v>
+      </c>
+      <c r="E589">
+        <v>600</v>
+      </c>
+      <c r="F589" t="s">
+        <v>10</v>
+      </c>
+      <c r="G589" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="590" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A590" t="s">
+        <v>89</v>
+      </c>
+      <c r="B590">
+        <v>6</v>
+      </c>
+      <c r="C590" t="s">
+        <v>92</v>
+      </c>
+      <c r="D590" t="s">
+        <v>93</v>
+      </c>
+      <c r="E590">
+        <v>960</v>
+      </c>
+      <c r="F590" t="s">
+        <v>10</v>
+      </c>
+      <c r="G590" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="591" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A591" t="s">
+        <v>89</v>
+      </c>
+      <c r="B591">
+        <v>6</v>
+      </c>
+      <c r="C591" t="s">
+        <v>64</v>
+      </c>
+      <c r="D591" t="s">
+        <v>65</v>
+      </c>
+      <c r="E591">
+        <v>300</v>
+      </c>
+      <c r="F591" t="s">
+        <v>10</v>
+      </c>
+      <c r="G591" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="592" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A592" t="s">
+        <v>89</v>
+      </c>
+      <c r="B592">
+        <v>6</v>
+      </c>
+      <c r="C592" t="s">
+        <v>68</v>
+      </c>
+      <c r="D592" t="s">
+        <v>69</v>
+      </c>
+      <c r="E592">
+        <v>270</v>
+      </c>
+      <c r="F592" t="s">
+        <v>10</v>
+      </c>
+      <c r="G592" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="593" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A593" t="s">
+        <v>187</v>
+      </c>
+      <c r="B593">
+        <v>6</v>
+      </c>
+      <c r="C593" t="s">
+        <v>58</v>
+      </c>
+      <c r="D593" t="s">
+        <v>59</v>
+      </c>
+      <c r="E593">
+        <v>1</v>
+      </c>
+      <c r="F593" t="s">
+        <v>15</v>
+      </c>
+      <c r="G593" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="594" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A594" t="s">
+        <v>187</v>
+      </c>
+      <c r="B594">
+        <v>6</v>
+      </c>
+      <c r="C594" t="s">
+        <v>60</v>
+      </c>
+      <c r="D594" t="s">
+        <v>61</v>
+      </c>
+      <c r="E594">
+        <v>234</v>
+      </c>
+      <c r="F594" t="s">
+        <v>10</v>
+      </c>
+      <c r="G594" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="595" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A595" t="s">
+        <v>187</v>
+      </c>
+      <c r="B595">
+        <v>6</v>
+      </c>
+      <c r="C595" t="s">
+        <v>62</v>
+      </c>
+      <c r="D595" t="s">
+        <v>63</v>
+      </c>
+      <c r="E595">
+        <v>150</v>
+      </c>
+      <c r="F595" t="s">
+        <v>10</v>
+      </c>
+      <c r="G595" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="596" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A596" t="s">
+        <v>187</v>
+      </c>
+      <c r="B596">
+        <v>6</v>
+      </c>
+      <c r="C596" t="s">
+        <v>64</v>
+      </c>
+      <c r="D596" t="s">
+        <v>65</v>
+      </c>
+      <c r="E596">
+        <v>90</v>
+      </c>
+      <c r="F596" t="s">
+        <v>10</v>
+      </c>
+      <c r="G596" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="597" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A597" t="s">
+        <v>187</v>
+      </c>
+      <c r="B597">
+        <v>6</v>
+      </c>
+      <c r="C597" t="s">
+        <v>53</v>
+      </c>
+      <c r="D597" t="s">
+        <v>54</v>
+      </c>
+      <c r="E597">
+        <v>4.8000000000000007</v>
+      </c>
+      <c r="F597" t="s">
+        <v>15</v>
+      </c>
+      <c r="G597" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="598" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A598" t="s">
+        <v>187</v>
+      </c>
+      <c r="B598">
+        <v>6</v>
+      </c>
+      <c r="C598" t="s">
+        <v>35</v>
+      </c>
+      <c r="D598" t="s">
+        <v>36</v>
+      </c>
+      <c r="E598">
+        <v>150</v>
+      </c>
+      <c r="F598" t="s">
+        <v>10</v>
+      </c>
+      <c r="G598" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="599" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A599" t="s">
+        <v>187</v>
+      </c>
+      <c r="B599">
+        <v>6</v>
+      </c>
+      <c r="C599" t="s">
+        <v>66</v>
+      </c>
+      <c r="D599" t="s">
+        <v>67</v>
+      </c>
+      <c r="E599">
+        <v>90</v>
+      </c>
+      <c r="F599" t="s">
+        <v>10</v>
+      </c>
+      <c r="G599" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="600" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A600" t="s">
+        <v>187</v>
+      </c>
+      <c r="B600">
+        <v>6</v>
+      </c>
+      <c r="C600" t="s">
+        <v>8</v>
+      </c>
+      <c r="D600" t="s">
+        <v>9</v>
+      </c>
+      <c r="E600">
+        <v>600</v>
+      </c>
+      <c r="F600" t="s">
+        <v>10</v>
+      </c>
+      <c r="G600" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="601" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A601" t="s">
+        <v>7</v>
+      </c>
+      <c r="B601">
+        <v>12</v>
+      </c>
+      <c r="C601" t="s">
+        <v>8</v>
+      </c>
+      <c r="D601" t="s">
+        <v>9</v>
+      </c>
+      <c r="E601">
+        <v>2100</v>
+      </c>
+      <c r="F601" t="s">
+        <v>10</v>
+      </c>
+      <c r="G601" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="602" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A602" t="s">
+        <v>7</v>
+      </c>
+      <c r="B602">
+        <v>12</v>
+      </c>
+      <c r="C602" t="s">
+        <v>11</v>
+      </c>
+      <c r="D602" t="s">
+        <v>12</v>
+      </c>
+      <c r="E602">
+        <v>2400</v>
+      </c>
+      <c r="F602" t="s">
+        <v>10</v>
+      </c>
+      <c r="G602" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="603" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A603" t="s">
+        <v>7</v>
+      </c>
+      <c r="B603">
+        <v>12</v>
+      </c>
+      <c r="C603" t="s">
+        <v>13</v>
+      </c>
+      <c r="D603" t="s">
+        <v>14</v>
+      </c>
+      <c r="E603">
+        <v>12</v>
+      </c>
+      <c r="F603" t="s">
+        <v>15</v>
+      </c>
+      <c r="G603" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="604" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A604" t="s">
+        <v>7</v>
+      </c>
+      <c r="B604">
+        <v>12</v>
+      </c>
+      <c r="C604" t="s">
+        <v>16</v>
+      </c>
+      <c r="D604" t="s">
+        <v>17</v>
+      </c>
+      <c r="E604">
+        <v>720</v>
+      </c>
+      <c r="F604" t="s">
+        <v>10</v>
+      </c>
+      <c r="G604" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="605" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A605" t="s">
+        <v>7</v>
+      </c>
+      <c r="B605">
+        <v>12</v>
+      </c>
+      <c r="C605" t="s">
+        <v>18</v>
+      </c>
+      <c r="D605" t="s">
+        <v>19</v>
+      </c>
+      <c r="E605">
+        <v>12</v>
+      </c>
+      <c r="F605" t="s">
+        <v>15</v>
+      </c>
+      <c r="G605" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="606" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A606" t="s">
+        <v>7</v>
+      </c>
+      <c r="B606">
+        <v>12</v>
+      </c>
+      <c r="C606" t="s">
+        <v>20</v>
+      </c>
+      <c r="D606" t="s">
+        <v>21</v>
+      </c>
+      <c r="E606">
+        <v>276</v>
+      </c>
+      <c r="F606" t="s">
+        <v>10</v>
+      </c>
+      <c r="G606" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="607" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A607" t="s">
+        <v>7</v>
+      </c>
+      <c r="B607">
+        <v>12</v>
+      </c>
+      <c r="C607" t="s">
+        <v>22</v>
+      </c>
+      <c r="D607" t="s">
+        <v>23</v>
+      </c>
+      <c r="E607">
+        <v>264</v>
+      </c>
+      <c r="F607" t="s">
+        <v>10</v>
+      </c>
+      <c r="G607" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="608" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A608" t="s">
+        <v>89</v>
+      </c>
+      <c r="B608">
+        <v>6</v>
+      </c>
+      <c r="C608" t="s">
+        <v>90</v>
+      </c>
+      <c r="D608" t="s">
+        <v>91</v>
+      </c>
+      <c r="E608">
+        <v>600</v>
+      </c>
+      <c r="F608" t="s">
+        <v>10</v>
+      </c>
+      <c r="G608" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="609" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A609" t="s">
+        <v>89</v>
+      </c>
+      <c r="B609">
+        <v>6</v>
+      </c>
+      <c r="C609" t="s">
+        <v>92</v>
+      </c>
+      <c r="D609" t="s">
+        <v>93</v>
+      </c>
+      <c r="E609">
+        <v>960</v>
+      </c>
+      <c r="F609" t="s">
+        <v>10</v>
+      </c>
+      <c r="G609" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="610" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A610" t="s">
+        <v>89</v>
+      </c>
+      <c r="B610">
+        <v>6</v>
+      </c>
+      <c r="C610" t="s">
+        <v>64</v>
+      </c>
+      <c r="D610" t="s">
+        <v>65</v>
+      </c>
+      <c r="E610">
+        <v>300</v>
+      </c>
+      <c r="F610" t="s">
+        <v>10</v>
+      </c>
+      <c r="G610" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="611" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A611" t="s">
+        <v>89</v>
+      </c>
+      <c r="B611">
+        <v>6</v>
+      </c>
+      <c r="C611" t="s">
+        <v>68</v>
+      </c>
+      <c r="D611" t="s">
+        <v>69</v>
+      </c>
+      <c r="E611">
+        <v>270</v>
+      </c>
+      <c r="F611" t="s">
+        <v>10</v>
+      </c>
+      <c r="G611" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="612" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A612" t="s">
+        <v>187</v>
+      </c>
+      <c r="B612">
+        <v>18</v>
+      </c>
+      <c r="C612" t="s">
+        <v>58</v>
+      </c>
+      <c r="D612" t="s">
+        <v>59</v>
+      </c>
+      <c r="E612">
+        <v>3</v>
+      </c>
+      <c r="F612" t="s">
+        <v>15</v>
+      </c>
+      <c r="G612" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="613" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A613" t="s">
+        <v>187</v>
+      </c>
+      <c r="B613">
+        <v>18</v>
+      </c>
+      <c r="C613" t="s">
+        <v>60</v>
+      </c>
+      <c r="D613" t="s">
+        <v>61</v>
+      </c>
+      <c r="E613">
+        <v>702</v>
+      </c>
+      <c r="F613" t="s">
+        <v>10</v>
+      </c>
+      <c r="G613" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="614" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A614" t="s">
+        <v>187</v>
+      </c>
+      <c r="B614">
+        <v>18</v>
+      </c>
+      <c r="C614" t="s">
+        <v>62</v>
+      </c>
+      <c r="D614" t="s">
+        <v>63</v>
+      </c>
+      <c r="E614">
+        <v>450</v>
+      </c>
+      <c r="F614" t="s">
+        <v>10</v>
+      </c>
+      <c r="G614" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="615" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A615" t="s">
+        <v>187</v>
+      </c>
+      <c r="B615">
+        <v>18</v>
+      </c>
+      <c r="C615" t="s">
+        <v>64</v>
+      </c>
+      <c r="D615" t="s">
+        <v>65</v>
+      </c>
+      <c r="E615">
+        <v>270</v>
+      </c>
+      <c r="F615" t="s">
+        <v>10</v>
+      </c>
+      <c r="G615" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="616" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A616" t="s">
+        <v>187</v>
+      </c>
+      <c r="B616">
+        <v>18</v>
+      </c>
+      <c r="C616" t="s">
+        <v>53</v>
+      </c>
+      <c r="D616" t="s">
+        <v>54</v>
+      </c>
+      <c r="E616">
+        <v>14.4</v>
+      </c>
+      <c r="F616" t="s">
+        <v>15</v>
+      </c>
+      <c r="G616" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="617" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A617" t="s">
+        <v>187</v>
+      </c>
+      <c r="B617">
+        <v>18</v>
+      </c>
+      <c r="C617" t="s">
+        <v>35</v>
+      </c>
+      <c r="D617" t="s">
+        <v>36</v>
+      </c>
+      <c r="E617">
+        <v>450</v>
+      </c>
+      <c r="F617" t="s">
+        <v>10</v>
+      </c>
+      <c r="G617" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="618" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A618" t="s">
+        <v>187</v>
+      </c>
+      <c r="B618">
+        <v>18</v>
+      </c>
+      <c r="C618" t="s">
+        <v>66</v>
+      </c>
+      <c r="D618" t="s">
+        <v>67</v>
+      </c>
+      <c r="E618">
+        <v>270</v>
+      </c>
+      <c r="F618" t="s">
+        <v>10</v>
+      </c>
+      <c r="G618" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="619" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A619" t="s">
+        <v>187</v>
+      </c>
+      <c r="B619">
+        <v>18</v>
+      </c>
+      <c r="C619" t="s">
+        <v>8</v>
+      </c>
+      <c r="D619" t="s">
+        <v>9</v>
+      </c>
+      <c r="E619">
+        <v>1800</v>
+      </c>
+      <c r="F619" t="s">
+        <v>10</v>
+      </c>
+      <c r="G619" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="620" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A620" t="s">
+        <v>7</v>
+      </c>
+      <c r="B620">
+        <v>13</v>
+      </c>
+      <c r="C620" t="s">
+        <v>8</v>
+      </c>
+      <c r="D620" t="s">
+        <v>9</v>
+      </c>
+      <c r="E620">
+        <v>2275</v>
+      </c>
+      <c r="F620" t="s">
+        <v>10</v>
+      </c>
+      <c r="G620" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="621" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A621" t="s">
+        <v>7</v>
+      </c>
+      <c r="B621">
+        <v>13</v>
+      </c>
+      <c r="C621" t="s">
+        <v>11</v>
+      </c>
+      <c r="D621" t="s">
+        <v>12</v>
+      </c>
+      <c r="E621">
+        <v>2600</v>
+      </c>
+      <c r="F621" t="s">
+        <v>10</v>
+      </c>
+      <c r="G621" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="622" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A622" t="s">
+        <v>7</v>
+      </c>
+      <c r="B622">
+        <v>13</v>
+      </c>
+      <c r="C622" t="s">
+        <v>13</v>
+      </c>
+      <c r="D622" t="s">
+        <v>14</v>
+      </c>
+      <c r="E622">
+        <v>13</v>
+      </c>
+      <c r="F622" t="s">
+        <v>15</v>
+      </c>
+      <c r="G622" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="623" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A623" t="s">
+        <v>7</v>
+      </c>
+      <c r="B623">
+        <v>13</v>
+      </c>
+      <c r="C623" t="s">
+        <v>16</v>
+      </c>
+      <c r="D623" t="s">
+        <v>17</v>
+      </c>
+      <c r="E623">
+        <v>780</v>
+      </c>
+      <c r="F623" t="s">
+        <v>10</v>
+      </c>
+      <c r="G623" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="624" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A624" t="s">
+        <v>7</v>
+      </c>
+      <c r="B624">
+        <v>13</v>
+      </c>
+      <c r="C624" t="s">
+        <v>18</v>
+      </c>
+      <c r="D624" t="s">
+        <v>19</v>
+      </c>
+      <c r="E624">
+        <v>13</v>
+      </c>
+      <c r="F624" t="s">
+        <v>15</v>
+      </c>
+      <c r="G624" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="625" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A625" t="s">
+        <v>7</v>
+      </c>
+      <c r="B625">
+        <v>13</v>
+      </c>
+      <c r="C625" t="s">
+        <v>20</v>
+      </c>
+      <c r="D625" t="s">
+        <v>21</v>
+      </c>
+      <c r="E625">
+        <v>299</v>
+      </c>
+      <c r="F625" t="s">
+        <v>10</v>
+      </c>
+      <c r="G625" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="626" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A626" t="s">
+        <v>7</v>
+      </c>
+      <c r="B626">
+        <v>13</v>
+      </c>
+      <c r="C626" t="s">
+        <v>22</v>
+      </c>
+      <c r="D626" t="s">
+        <v>23</v>
+      </c>
+      <c r="E626">
+        <v>286</v>
+      </c>
+      <c r="F626" t="s">
+        <v>10</v>
+      </c>
+      <c r="G626" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="627" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A627" t="s">
+        <v>89</v>
+      </c>
+      <c r="B627">
+        <v>3</v>
+      </c>
+      <c r="C627" t="s">
+        <v>90</v>
+      </c>
+      <c r="D627" t="s">
+        <v>91</v>
+      </c>
+      <c r="E627">
+        <v>300</v>
+      </c>
+      <c r="F627" t="s">
+        <v>10</v>
+      </c>
+      <c r="G627" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="628" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A628" t="s">
+        <v>89</v>
+      </c>
+      <c r="B628">
+        <v>3</v>
+      </c>
+      <c r="C628" t="s">
+        <v>92</v>
+      </c>
+      <c r="D628" t="s">
+        <v>93</v>
+      </c>
+      <c r="E628">
+        <v>480</v>
+      </c>
+      <c r="F628" t="s">
+        <v>10</v>
+      </c>
+      <c r="G628" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="629" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A629" t="s">
+        <v>89</v>
+      </c>
+      <c r="B629">
+        <v>3</v>
+      </c>
+      <c r="C629" t="s">
+        <v>64</v>
+      </c>
+      <c r="D629" t="s">
+        <v>65</v>
+      </c>
+      <c r="E629">
+        <v>150</v>
+      </c>
+      <c r="F629" t="s">
+        <v>10</v>
+      </c>
+      <c r="G629" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="630" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A630" t="s">
+        <v>89</v>
+      </c>
+      <c r="B630">
+        <v>3</v>
+      </c>
+      <c r="C630" t="s">
+        <v>68</v>
+      </c>
+      <c r="D630" t="s">
+        <v>69</v>
+      </c>
+      <c r="E630">
+        <v>135</v>
+      </c>
+      <c r="F630" t="s">
+        <v>10</v>
+      </c>
+      <c r="G630" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="631" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G631" s="2"/>
+    </row>
+    <row r="632" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G632" s="2"/>
+    </row>
+    <row r="633" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G633" s="2"/>
+    </row>
+    <row r="634" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G634" s="2"/>
+    </row>
+    <row r="635" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G635" s="2"/>
+    </row>
+    <row r="636" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G636" s="2"/>
+    </row>
+    <row r="637" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G637" s="2"/>
+    </row>
+    <row r="638" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G638" s="2"/>
+    </row>
+    <row r="639" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G639" s="2"/>
+    </row>
+    <row r="640" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G640" s="2"/>
+    </row>
+    <row r="641" spans="7:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G641" s="2"/>
+    </row>
+    <row r="642" spans="7:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G642" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -14955,7 +15955,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D567"/>
+  <dimension ref="A1:D644"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="14.68359375" bestFit="1" customWidth="1"/>
@@ -22439,13 +23439,13 @@
       </c>
     </row>
     <row r="535" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A535" s="5" t="s">
+      <c r="A535" t="s">
         <v>101</v>
       </c>
-      <c r="B535" s="5">
+      <c r="B535">
         <v>1</v>
       </c>
-      <c r="C535" s="5" t="s">
+      <c r="C535" t="s">
         <v>15</v>
       </c>
       <c r="D535" s="2">
@@ -22453,13 +23453,13 @@
       </c>
     </row>
     <row r="536" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A536" s="5" t="s">
+      <c r="A536" t="s">
         <v>102</v>
       </c>
-      <c r="B536" s="5">
+      <c r="B536">
         <v>16</v>
       </c>
-      <c r="C536" s="5" t="s">
+      <c r="C536" t="s">
         <v>15</v>
       </c>
       <c r="D536" s="2">
@@ -22467,13 +23467,13 @@
       </c>
     </row>
     <row r="537" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A537" s="5" t="s">
+      <c r="A537" t="s">
         <v>39</v>
       </c>
-      <c r="B537" s="5">
+      <c r="B537">
         <v>2.04</v>
       </c>
-      <c r="C537" s="5" t="s">
+      <c r="C537" t="s">
         <v>15</v>
       </c>
       <c r="D537" s="2">
@@ -22481,13 +23481,13 @@
       </c>
     </row>
     <row r="538" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A538" s="5" t="s">
+      <c r="A538" t="s">
         <v>94</v>
       </c>
-      <c r="B538" s="5">
+      <c r="B538">
         <v>1</v>
       </c>
-      <c r="C538" s="5" t="s">
+      <c r="C538" t="s">
         <v>15</v>
       </c>
       <c r="D538" s="2">
@@ -22495,13 +23495,13 @@
       </c>
     </row>
     <row r="539" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A539" s="5" t="s">
+      <c r="A539" t="s">
         <v>76</v>
       </c>
-      <c r="B539" s="5">
+      <c r="B539">
         <v>200</v>
       </c>
-      <c r="C539" s="5" t="s">
+      <c r="C539" t="s">
         <v>10</v>
       </c>
       <c r="D539" s="2">
@@ -22509,13 +23509,13 @@
       </c>
     </row>
     <row r="540" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A540" s="5" t="s">
+      <c r="A540" t="s">
         <v>35</v>
       </c>
-      <c r="B540" s="5">
+      <c r="B540">
         <v>768</v>
       </c>
-      <c r="C540" s="5" t="s">
+      <c r="C540" t="s">
         <v>10</v>
       </c>
       <c r="D540" s="2">
@@ -22523,13 +23523,13 @@
       </c>
     </row>
     <row r="541" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A541" s="5" t="s">
+      <c r="A541" t="s">
         <v>37</v>
       </c>
-      <c r="B541" s="5">
+      <c r="B541">
         <v>3</v>
       </c>
-      <c r="C541" s="5" t="s">
+      <c r="C541" t="s">
         <v>15</v>
       </c>
       <c r="D541" s="2">
@@ -22537,13 +23537,13 @@
       </c>
     </row>
     <row r="542" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A542" s="5" t="s">
+      <c r="A542" t="s">
         <v>95</v>
       </c>
-      <c r="B542" s="5">
+      <c r="B542">
         <v>1</v>
       </c>
-      <c r="C542" s="5" t="s">
+      <c r="C542" t="s">
         <v>15</v>
       </c>
       <c r="D542" s="2">
@@ -22551,13 +23551,13 @@
       </c>
     </row>
     <row r="543" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A543" s="5" t="s">
+      <c r="A543" t="s">
         <v>43</v>
       </c>
-      <c r="B543" s="5">
+      <c r="B543">
         <v>1800</v>
       </c>
-      <c r="C543" s="5" t="s">
+      <c r="C543" t="s">
         <v>10</v>
       </c>
       <c r="D543" s="2">
@@ -22565,13 +23565,13 @@
       </c>
     </row>
     <row r="544" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A544" s="5" t="s">
+      <c r="A544" t="s">
         <v>53</v>
       </c>
-      <c r="B544" s="5">
+      <c r="B544">
         <v>40</v>
       </c>
-      <c r="C544" s="5" t="s">
+      <c r="C544" t="s">
         <v>15</v>
       </c>
       <c r="D544" s="2">
@@ -22579,13 +23579,13 @@
       </c>
     </row>
     <row r="545" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A545" s="5" t="s">
+      <c r="A545" t="s">
         <v>28</v>
       </c>
-      <c r="B545" s="5">
+      <c r="B545">
         <v>400</v>
       </c>
-      <c r="C545" s="5" t="s">
+      <c r="C545" t="s">
         <v>10</v>
       </c>
       <c r="D545" s="2">
@@ -22593,13 +23593,13 @@
       </c>
     </row>
     <row r="546" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A546" s="5" t="s">
+      <c r="A546" t="s">
         <v>178</v>
       </c>
-      <c r="B546" s="5">
+      <c r="B546">
         <v>1</v>
       </c>
-      <c r="C546" s="5" t="s">
+      <c r="C546" t="s">
         <v>15</v>
       </c>
       <c r="D546" s="2">
@@ -22607,13 +23607,13 @@
       </c>
     </row>
     <row r="547" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A547" s="5" t="s">
+      <c r="A547" t="s">
         <v>78</v>
       </c>
-      <c r="B547" s="5">
+      <c r="B547">
         <v>8</v>
       </c>
-      <c r="C547" s="5" t="s">
+      <c r="C547" t="s">
         <v>10</v>
       </c>
       <c r="D547" s="2">
@@ -22621,13 +23621,13 @@
       </c>
     </row>
     <row r="548" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A548" s="5" t="s">
+      <c r="A548" t="s">
         <v>72</v>
       </c>
-      <c r="B548" s="5">
+      <c r="B548">
         <v>1000</v>
       </c>
-      <c r="C548" s="5" t="s">
+      <c r="C548" t="s">
         <v>10</v>
       </c>
       <c r="D548" s="2">
@@ -22635,13 +23635,13 @@
       </c>
     </row>
     <row r="549" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A549" s="5" t="s">
+      <c r="A549" t="s">
         <v>47</v>
       </c>
-      <c r="B549" s="5">
+      <c r="B549">
         <v>150</v>
       </c>
-      <c r="C549" s="5" t="s">
+      <c r="C549" t="s">
         <v>10</v>
       </c>
       <c r="D549" s="2">
@@ -22649,13 +23649,13 @@
       </c>
     </row>
     <row r="550" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A550" s="5" t="s">
+      <c r="A550" t="s">
         <v>18</v>
       </c>
-      <c r="B550" s="5">
+      <c r="B550">
         <v>16</v>
       </c>
-      <c r="C550" s="5" t="s">
+      <c r="C550" t="s">
         <v>15</v>
       </c>
       <c r="D550" s="2">
@@ -22663,13 +23663,13 @@
       </c>
     </row>
     <row r="551" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A551" s="5" t="s">
+      <c r="A551" t="s">
         <v>45</v>
       </c>
-      <c r="B551" s="5">
+      <c r="B551">
         <v>120</v>
       </c>
-      <c r="C551" s="5" t="s">
+      <c r="C551" t="s">
         <v>10</v>
       </c>
       <c r="D551" s="2">
@@ -22677,13 +23677,13 @@
       </c>
     </row>
     <row r="552" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A552" s="5" t="s">
+      <c r="A552" t="s">
         <v>55</v>
       </c>
-      <c r="B552" s="5">
+      <c r="B552">
         <v>120</v>
       </c>
-      <c r="C552" s="5" t="s">
+      <c r="C552" t="s">
         <v>10</v>
       </c>
       <c r="D552" s="2">
@@ -22691,13 +23691,13 @@
       </c>
     </row>
     <row r="553" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A553" s="5" t="s">
+      <c r="A553" t="s">
         <v>55</v>
       </c>
-      <c r="B553" s="5">
+      <c r="B553">
         <v>4</v>
       </c>
-      <c r="C553" s="5" t="s">
+      <c r="C553" t="s">
         <v>15</v>
       </c>
       <c r="D553" s="2">
@@ -22705,13 +23705,13 @@
       </c>
     </row>
     <row r="554" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A554" s="5" t="s">
+      <c r="A554" t="s">
         <v>64</v>
       </c>
-      <c r="B554" s="5">
+      <c r="B554">
         <v>300</v>
       </c>
-      <c r="C554" s="5" t="s">
+      <c r="C554" t="s">
         <v>10</v>
       </c>
       <c r="D554" s="2">
@@ -22719,13 +23719,13 @@
       </c>
     </row>
     <row r="555" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A555" s="5" t="s">
+      <c r="A555" t="s">
         <v>140</v>
       </c>
-      <c r="B555" s="5">
+      <c r="B555">
         <v>1</v>
       </c>
-      <c r="C555" s="5" t="s">
+      <c r="C555" t="s">
         <v>15</v>
       </c>
       <c r="D555" s="2">
@@ -22733,13 +23733,13 @@
       </c>
     </row>
     <row r="556" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A556" s="5" t="s">
+      <c r="A556" t="s">
         <v>16</v>
       </c>
-      <c r="B556" s="5">
+      <c r="B556">
         <v>720</v>
       </c>
-      <c r="C556" s="5" t="s">
+      <c r="C556" t="s">
         <v>10</v>
       </c>
       <c r="D556" s="2">
@@ -22747,13 +23747,13 @@
       </c>
     </row>
     <row r="557" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A557" s="5" t="s">
+      <c r="A557" t="s">
         <v>24</v>
       </c>
-      <c r="B557" s="5">
+      <c r="B557">
         <v>3</v>
       </c>
-      <c r="C557" s="5" t="s">
+      <c r="C557" t="s">
         <v>15</v>
       </c>
       <c r="D557" s="2">
@@ -22761,13 +23761,13 @@
       </c>
     </row>
     <row r="558" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A558" s="5" t="s">
+      <c r="A558" t="s">
         <v>74</v>
       </c>
-      <c r="B558" s="5">
+      <c r="B558">
         <v>400</v>
       </c>
-      <c r="C558" s="5" t="s">
+      <c r="C558" t="s">
         <v>10</v>
       </c>
       <c r="D558" s="2">
@@ -22775,13 +23775,13 @@
       </c>
     </row>
     <row r="559" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A559" s="5" t="s">
+      <c r="A559" t="s">
         <v>68</v>
       </c>
-      <c r="B559" s="5">
+      <c r="B559">
         <v>270</v>
       </c>
-      <c r="C559" s="5" t="s">
+      <c r="C559" t="s">
         <v>10</v>
       </c>
       <c r="D559" s="2">
@@ -22789,13 +23789,13 @@
       </c>
     </row>
     <row r="560" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A560" s="5" t="s">
+      <c r="A560" t="s">
         <v>96</v>
       </c>
-      <c r="B560" s="5">
+      <c r="B560">
         <v>4</v>
       </c>
-      <c r="C560" s="5" t="s">
+      <c r="C560" t="s">
         <v>15</v>
       </c>
       <c r="D560" s="2">
@@ -22803,13 +23803,13 @@
       </c>
     </row>
     <row r="561" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A561" s="5" t="s">
+      <c r="A561" t="s">
         <v>109</v>
       </c>
-      <c r="B561" s="5">
+      <c r="B561">
         <v>4</v>
       </c>
-      <c r="C561" s="5" t="s">
+      <c r="C561" t="s">
         <v>15</v>
       </c>
       <c r="D561" s="2">
@@ -22817,13 +23817,13 @@
       </c>
     </row>
     <row r="562" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A562" s="5" t="s">
+      <c r="A562" t="s">
         <v>20</v>
       </c>
-      <c r="B562" s="5">
+      <c r="B562">
         <v>150</v>
       </c>
-      <c r="C562" s="5" t="s">
+      <c r="C562" t="s">
         <v>10</v>
       </c>
       <c r="D562" s="2">
@@ -22831,13 +23831,13 @@
       </c>
     </row>
     <row r="563" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A563" s="5" t="s">
+      <c r="A563" t="s">
         <v>90</v>
       </c>
-      <c r="B563" s="5">
+      <c r="B563">
         <v>600</v>
       </c>
-      <c r="C563" s="5" t="s">
+      <c r="C563" t="s">
         <v>10</v>
       </c>
       <c r="D563" s="2">
@@ -22845,13 +23845,13 @@
       </c>
     </row>
     <row r="564" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A564" s="5" t="s">
+      <c r="A564" t="s">
         <v>92</v>
       </c>
-      <c r="B564" s="5">
+      <c r="B564">
         <v>960</v>
       </c>
-      <c r="C564" s="5" t="s">
+      <c r="C564" t="s">
         <v>10</v>
       </c>
       <c r="D564" s="2">
@@ -22859,13 +23859,13 @@
       </c>
     </row>
     <row r="565" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A565" s="5" t="s">
+      <c r="A565" t="s">
         <v>8</v>
       </c>
-      <c r="B565" s="5">
+      <c r="B565">
         <v>600</v>
       </c>
-      <c r="C565" s="5" t="s">
+      <c r="C565" t="s">
         <v>10</v>
       </c>
       <c r="D565" s="2">
@@ -22873,13 +23873,13 @@
       </c>
     </row>
     <row r="566" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A566" s="5" t="s">
+      <c r="A566" t="s">
         <v>97</v>
       </c>
-      <c r="B566" s="5">
+      <c r="B566">
         <v>2</v>
       </c>
-      <c r="C566" s="5" t="s">
+      <c r="C566" t="s">
         <v>15</v>
       </c>
       <c r="D566" s="2">
@@ -22887,17 +23887,1095 @@
       </c>
     </row>
     <row r="567" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A567" s="5" t="s">
+      <c r="A567" t="s">
         <v>41</v>
       </c>
-      <c r="B567" s="5">
+      <c r="B567">
         <v>6</v>
       </c>
-      <c r="C567" s="5" t="s">
+      <c r="C567" t="s">
         <v>15</v>
       </c>
       <c r="D567" s="2">
         <v>45918</v>
+      </c>
+    </row>
+    <row r="568" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A568" t="s">
+        <v>101</v>
+      </c>
+      <c r="B568">
+        <v>1</v>
+      </c>
+      <c r="C568" t="s">
+        <v>15</v>
+      </c>
+      <c r="D568" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="569" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A569" t="s">
+        <v>102</v>
+      </c>
+      <c r="B569">
+        <v>22</v>
+      </c>
+      <c r="C569" t="s">
+        <v>15</v>
+      </c>
+      <c r="D569" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="570" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A570" t="s">
+        <v>94</v>
+      </c>
+      <c r="B570">
+        <v>1</v>
+      </c>
+      <c r="C570" t="s">
+        <v>15</v>
+      </c>
+      <c r="D570" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="571" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A571" t="s">
+        <v>58</v>
+      </c>
+      <c r="B571">
+        <v>1</v>
+      </c>
+      <c r="C571" t="s">
+        <v>15</v>
+      </c>
+      <c r="D571" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="572" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A572" t="s">
+        <v>11</v>
+      </c>
+      <c r="B572">
+        <v>2400</v>
+      </c>
+      <c r="C572" t="s">
+        <v>10</v>
+      </c>
+      <c r="D572" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="573" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A573" t="s">
+        <v>35</v>
+      </c>
+      <c r="B573">
+        <v>150</v>
+      </c>
+      <c r="C573" t="s">
+        <v>10</v>
+      </c>
+      <c r="D573" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="574" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A574" t="s">
+        <v>95</v>
+      </c>
+      <c r="B574">
+        <v>2</v>
+      </c>
+      <c r="C574" t="s">
+        <v>15</v>
+      </c>
+      <c r="D574" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="575" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A575" t="s">
+        <v>43</v>
+      </c>
+      <c r="B575">
+        <v>1350</v>
+      </c>
+      <c r="C575" t="s">
+        <v>10</v>
+      </c>
+      <c r="D575" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="576" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A576" t="s">
+        <v>53</v>
+      </c>
+      <c r="B576">
+        <v>44.8</v>
+      </c>
+      <c r="C576" t="s">
+        <v>15</v>
+      </c>
+      <c r="D576" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="577" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A577" t="s">
+        <v>178</v>
+      </c>
+      <c r="B577">
+        <v>1</v>
+      </c>
+      <c r="C577" t="s">
+        <v>15</v>
+      </c>
+      <c r="D577" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="578" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A578" t="s">
+        <v>141</v>
+      </c>
+      <c r="B578">
+        <v>1</v>
+      </c>
+      <c r="C578" t="s">
+        <v>15</v>
+      </c>
+      <c r="D578" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="579" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A579" t="s">
+        <v>105</v>
+      </c>
+      <c r="B579">
+        <v>1</v>
+      </c>
+      <c r="C579" t="s">
+        <v>15</v>
+      </c>
+      <c r="D579" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="580" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A580" t="s">
+        <v>72</v>
+      </c>
+      <c r="B580">
+        <v>1</v>
+      </c>
+      <c r="C580" t="s">
+        <v>15</v>
+      </c>
+      <c r="D580" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="581" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A581" t="s">
+        <v>18</v>
+      </c>
+      <c r="B581">
+        <v>12</v>
+      </c>
+      <c r="C581" t="s">
+        <v>15</v>
+      </c>
+      <c r="D581" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="582" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A582" t="s">
+        <v>13</v>
+      </c>
+      <c r="B582">
+        <v>12</v>
+      </c>
+      <c r="C582" t="s">
+        <v>15</v>
+      </c>
+      <c r="D582" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="583" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A583" t="s">
+        <v>106</v>
+      </c>
+      <c r="B583">
+        <v>12</v>
+      </c>
+      <c r="C583" t="s">
+        <v>15</v>
+      </c>
+      <c r="D583" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="584" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A584" t="s">
+        <v>55</v>
+      </c>
+      <c r="B584">
+        <v>4</v>
+      </c>
+      <c r="C584" t="s">
+        <v>15</v>
+      </c>
+      <c r="D584" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="585" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A585" t="s">
+        <v>22</v>
+      </c>
+      <c r="B585">
+        <v>264</v>
+      </c>
+      <c r="C585" t="s">
+        <v>10</v>
+      </c>
+      <c r="D585" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="586" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A586" t="s">
+        <v>66</v>
+      </c>
+      <c r="B586">
+        <v>90</v>
+      </c>
+      <c r="C586" t="s">
+        <v>10</v>
+      </c>
+      <c r="D586" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="587" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A587" t="s">
+        <v>64</v>
+      </c>
+      <c r="B587">
+        <v>390</v>
+      </c>
+      <c r="C587" t="s">
+        <v>10</v>
+      </c>
+      <c r="D587" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="588" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A588" t="s">
+        <v>140</v>
+      </c>
+      <c r="B588">
+        <v>1</v>
+      </c>
+      <c r="C588" t="s">
+        <v>15</v>
+      </c>
+      <c r="D588" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="589" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A589" t="s">
+        <v>60</v>
+      </c>
+      <c r="B589">
+        <v>234</v>
+      </c>
+      <c r="C589" t="s">
+        <v>10</v>
+      </c>
+      <c r="D589" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="590" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A590" t="s">
+        <v>16</v>
+      </c>
+      <c r="B590">
+        <v>720</v>
+      </c>
+      <c r="C590" t="s">
+        <v>10</v>
+      </c>
+      <c r="D590" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="591" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A591" t="s">
+        <v>68</v>
+      </c>
+      <c r="B591">
+        <v>270</v>
+      </c>
+      <c r="C591" t="s">
+        <v>10</v>
+      </c>
+      <c r="D591" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="592" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A592" t="s">
+        <v>96</v>
+      </c>
+      <c r="B592">
+        <v>4</v>
+      </c>
+      <c r="C592" t="s">
+        <v>15</v>
+      </c>
+      <c r="D592" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="593" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A593" t="s">
+        <v>109</v>
+      </c>
+      <c r="B593">
+        <v>4</v>
+      </c>
+      <c r="C593" t="s">
+        <v>15</v>
+      </c>
+      <c r="D593" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="594" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A594" t="s">
+        <v>20</v>
+      </c>
+      <c r="B594">
+        <v>276</v>
+      </c>
+      <c r="C594" t="s">
+        <v>10</v>
+      </c>
+      <c r="D594" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="595" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A595" t="s">
+        <v>90</v>
+      </c>
+      <c r="B595">
+        <v>600</v>
+      </c>
+      <c r="C595" t="s">
+        <v>10</v>
+      </c>
+      <c r="D595" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="596" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A596" t="s">
+        <v>92</v>
+      </c>
+      <c r="B596">
+        <v>960</v>
+      </c>
+      <c r="C596" t="s">
+        <v>10</v>
+      </c>
+      <c r="D596" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="597" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A597" t="s">
+        <v>8</v>
+      </c>
+      <c r="B597">
+        <v>2700</v>
+      </c>
+      <c r="C597" t="s">
+        <v>10</v>
+      </c>
+      <c r="D597" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="598" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A598" t="s">
+        <v>97</v>
+      </c>
+      <c r="B598">
+        <v>2</v>
+      </c>
+      <c r="C598" t="s">
+        <v>15</v>
+      </c>
+      <c r="D598" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="599" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A599" t="s">
+        <v>62</v>
+      </c>
+      <c r="B599">
+        <v>150</v>
+      </c>
+      <c r="C599" t="s">
+        <v>10</v>
+      </c>
+      <c r="D599" s="2">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="600" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A600" t="s">
+        <v>101</v>
+      </c>
+      <c r="B600">
+        <v>1</v>
+      </c>
+      <c r="C600" t="s">
+        <v>15</v>
+      </c>
+      <c r="D600" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="601" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A601" t="s">
+        <v>102</v>
+      </c>
+      <c r="B601">
+        <v>18</v>
+      </c>
+      <c r="C601" t="s">
+        <v>15</v>
+      </c>
+      <c r="D601" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="602" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A602" t="s">
+        <v>94</v>
+      </c>
+      <c r="B602">
+        <v>1</v>
+      </c>
+      <c r="C602" t="s">
+        <v>15</v>
+      </c>
+      <c r="D602" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="603" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A603" t="s">
+        <v>58</v>
+      </c>
+      <c r="B603">
+        <v>3</v>
+      </c>
+      <c r="C603" t="s">
+        <v>15</v>
+      </c>
+      <c r="D603" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="604" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A604" t="s">
+        <v>35</v>
+      </c>
+      <c r="B604">
+        <v>450</v>
+      </c>
+      <c r="C604" t="s">
+        <v>10</v>
+      </c>
+      <c r="D604" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="605" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A605" t="s">
+        <v>95</v>
+      </c>
+      <c r="B605">
+        <v>1</v>
+      </c>
+      <c r="C605" t="s">
+        <v>15</v>
+      </c>
+      <c r="D605" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="606" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A606" t="s">
+        <v>43</v>
+      </c>
+      <c r="B606">
+        <v>1350</v>
+      </c>
+      <c r="C606" t="s">
+        <v>10</v>
+      </c>
+      <c r="D606" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="607" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A607" t="s">
+        <v>53</v>
+      </c>
+      <c r="B607">
+        <v>54.4</v>
+      </c>
+      <c r="C607" t="s">
+        <v>15</v>
+      </c>
+      <c r="D607" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="608" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A608" t="s">
+        <v>55</v>
+      </c>
+      <c r="B608">
+        <v>4</v>
+      </c>
+      <c r="C608" t="s">
+        <v>15</v>
+      </c>
+      <c r="D608" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="609" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A609" t="s">
+        <v>66</v>
+      </c>
+      <c r="B609">
+        <v>270</v>
+      </c>
+      <c r="C609" t="s">
+        <v>10</v>
+      </c>
+      <c r="D609" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="610" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A610" t="s">
+        <v>64</v>
+      </c>
+      <c r="B610">
+        <v>570</v>
+      </c>
+      <c r="C610" t="s">
+        <v>10</v>
+      </c>
+      <c r="D610" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="611" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A611" t="s">
+        <v>140</v>
+      </c>
+      <c r="B611">
+        <v>1</v>
+      </c>
+      <c r="C611" t="s">
+        <v>15</v>
+      </c>
+      <c r="D611" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="612" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A612" t="s">
+        <v>60</v>
+      </c>
+      <c r="B612">
+        <v>702</v>
+      </c>
+      <c r="C612" t="s">
+        <v>10</v>
+      </c>
+      <c r="D612" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="613" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A613" t="s">
+        <v>68</v>
+      </c>
+      <c r="B613">
+        <v>270</v>
+      </c>
+      <c r="C613" t="s">
+        <v>10</v>
+      </c>
+      <c r="D613" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="614" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A614" t="s">
+        <v>96</v>
+      </c>
+      <c r="B614">
+        <v>4</v>
+      </c>
+      <c r="C614" t="s">
+        <v>15</v>
+      </c>
+      <c r="D614" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="615" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A615" t="s">
+        <v>109</v>
+      </c>
+      <c r="B615">
+        <v>4</v>
+      </c>
+      <c r="C615" t="s">
+        <v>15</v>
+      </c>
+      <c r="D615" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="616" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A616" t="s">
+        <v>90</v>
+      </c>
+      <c r="B616">
+        <v>600</v>
+      </c>
+      <c r="C616" t="s">
+        <v>10</v>
+      </c>
+      <c r="D616" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="617" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A617" t="s">
+        <v>92</v>
+      </c>
+      <c r="B617">
+        <v>960</v>
+      </c>
+      <c r="C617" t="s">
+        <v>10</v>
+      </c>
+      <c r="D617" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="618" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A618" t="s">
+        <v>8</v>
+      </c>
+      <c r="B618">
+        <v>1800</v>
+      </c>
+      <c r="C618" t="s">
+        <v>10</v>
+      </c>
+      <c r="D618" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="619" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A619" t="s">
+        <v>97</v>
+      </c>
+      <c r="B619">
+        <v>2</v>
+      </c>
+      <c r="C619" t="s">
+        <v>15</v>
+      </c>
+      <c r="D619" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="620" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A620" t="s">
+        <v>62</v>
+      </c>
+      <c r="B620">
+        <v>450</v>
+      </c>
+      <c r="C620" t="s">
+        <v>10</v>
+      </c>
+      <c r="D620" s="2">
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="621" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A621" t="s">
+        <v>101</v>
+      </c>
+      <c r="B621">
+        <v>1</v>
+      </c>
+      <c r="C621" t="s">
+        <v>15</v>
+      </c>
+      <c r="D621" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="622" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A622" t="s">
+        <v>102</v>
+      </c>
+      <c r="B622">
+        <v>16</v>
+      </c>
+      <c r="C622" t="s">
+        <v>15</v>
+      </c>
+      <c r="D622" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="623" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A623" t="s">
+        <v>94</v>
+      </c>
+      <c r="B623">
+        <v>2</v>
+      </c>
+      <c r="C623" t="s">
+        <v>15</v>
+      </c>
+      <c r="D623" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="624" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A624" t="s">
+        <v>11</v>
+      </c>
+      <c r="B624">
+        <v>2600</v>
+      </c>
+      <c r="C624" t="s">
+        <v>10</v>
+      </c>
+      <c r="D624" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="625" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A625" t="s">
+        <v>95</v>
+      </c>
+      <c r="B625">
+        <v>2</v>
+      </c>
+      <c r="C625" t="s">
+        <v>15</v>
+      </c>
+      <c r="D625" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="626" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A626" t="s">
+        <v>43</v>
+      </c>
+      <c r="B626">
+        <v>1200</v>
+      </c>
+      <c r="C626" t="s">
+        <v>10</v>
+      </c>
+      <c r="D626" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="627" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A627" t="s">
+        <v>53</v>
+      </c>
+      <c r="B627">
+        <v>36</v>
+      </c>
+      <c r="C627" t="s">
+        <v>15</v>
+      </c>
+      <c r="D627" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="628" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A628" t="s">
+        <v>178</v>
+      </c>
+      <c r="B628">
+        <v>1</v>
+      </c>
+      <c r="C628" t="s">
+        <v>15</v>
+      </c>
+      <c r="D628" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="629" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A629" t="s">
+        <v>18</v>
+      </c>
+      <c r="B629">
+        <v>13</v>
+      </c>
+      <c r="C629" t="s">
+        <v>15</v>
+      </c>
+      <c r="D629" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="630" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A630" t="s">
+        <v>13</v>
+      </c>
+      <c r="B630">
+        <v>13</v>
+      </c>
+      <c r="C630" t="s">
+        <v>15</v>
+      </c>
+      <c r="D630" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="631" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A631" t="s">
+        <v>106</v>
+      </c>
+      <c r="B631">
+        <v>16</v>
+      </c>
+      <c r="C631" t="s">
+        <v>15</v>
+      </c>
+      <c r="D631" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="632" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A632" t="s">
+        <v>55</v>
+      </c>
+      <c r="B632">
+        <v>4</v>
+      </c>
+      <c r="C632" t="s">
+        <v>15</v>
+      </c>
+      <c r="D632" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="633" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A633" t="s">
+        <v>22</v>
+      </c>
+      <c r="B633">
+        <v>286</v>
+      </c>
+      <c r="C633" t="s">
+        <v>10</v>
+      </c>
+      <c r="D633" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="634" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A634" t="s">
+        <v>64</v>
+      </c>
+      <c r="B634">
+        <v>150</v>
+      </c>
+      <c r="C634" t="s">
+        <v>10</v>
+      </c>
+      <c r="D634" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="635" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A635" t="s">
+        <v>16</v>
+      </c>
+      <c r="B635">
+        <v>780</v>
+      </c>
+      <c r="C635" t="s">
+        <v>10</v>
+      </c>
+      <c r="D635" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="636" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A636" t="s">
+        <v>68</v>
+      </c>
+      <c r="B636">
+        <v>135</v>
+      </c>
+      <c r="C636" t="s">
+        <v>10</v>
+      </c>
+      <c r="D636" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="637" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A637" t="s">
+        <v>96</v>
+      </c>
+      <c r="B637">
+        <v>4</v>
+      </c>
+      <c r="C637" t="s">
+        <v>15</v>
+      </c>
+      <c r="D637" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="638" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A638" t="s">
+        <v>109</v>
+      </c>
+      <c r="B638">
+        <v>4</v>
+      </c>
+      <c r="C638" t="s">
+        <v>15</v>
+      </c>
+      <c r="D638" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="639" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A639" t="s">
+        <v>20</v>
+      </c>
+      <c r="B639">
+        <v>299</v>
+      </c>
+      <c r="C639" t="s">
+        <v>10</v>
+      </c>
+      <c r="D639" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="640" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A640" t="s">
+        <v>90</v>
+      </c>
+      <c r="B640">
+        <v>300</v>
+      </c>
+      <c r="C640" t="s">
+        <v>10</v>
+      </c>
+      <c r="D640" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="641" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A641" t="s">
+        <v>92</v>
+      </c>
+      <c r="B641">
+        <v>480</v>
+      </c>
+      <c r="C641" t="s">
+        <v>10</v>
+      </c>
+      <c r="D641" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="642" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A642" t="s">
+        <v>8</v>
+      </c>
+      <c r="B642">
+        <v>2275</v>
+      </c>
+      <c r="C642" t="s">
+        <v>10</v>
+      </c>
+      <c r="D642" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="643" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A643" t="s">
+        <v>97</v>
+      </c>
+      <c r="B643">
+        <v>2</v>
+      </c>
+      <c r="C643" t="s">
+        <v>15</v>
+      </c>
+      <c r="D643" s="2">
+        <v>45943</v>
+      </c>
+    </row>
+    <row r="644" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A644" t="s">
+        <v>142</v>
+      </c>
+      <c r="B644">
+        <v>6</v>
+      </c>
+      <c r="C644" t="s">
+        <v>15</v>
+      </c>
+      <c r="D644" s="2">
+        <v>45943</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New Export 21 09 2026
</commit_message>
<xml_diff>
--- a/Excel_files/Log/Grocery_List_Log.xlsx
+++ b/Excel_files/Log/Grocery_List_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Grocery_list\Excel_files\Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5425CD34-C824-4A1B-8343-04D7405D73F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62FE357D-18DB-4470-9AE6-BEC67915767F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="1560" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="1560" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Log Per Recipe" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4050" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4040" uniqueCount="190">
   <si>
     <t>Recipe</t>
   </si>
@@ -594,18 +594,6 @@
   </si>
   <si>
     <t>Nectarine (Wit)</t>
-  </si>
-  <si>
-    <t>Rozijnen</t>
-  </si>
-  <si>
-    <t>SKYR</t>
-  </si>
-  <si>
-    <t>ROZIJNEN</t>
-  </si>
-  <si>
-    <t>ZALM&amp;EIGENSALADE</t>
   </si>
   <si>
     <t>Yakult</t>
@@ -15926,22 +15914,22 @@
     </row>
     <row r="631" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A631" t="s">
-        <v>89</v>
+        <v>136</v>
       </c>
       <c r="B631">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C631" t="s">
-        <v>90</v>
+        <v>133</v>
       </c>
       <c r="D631" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="E631">
-        <v>300</v>
+        <v>2</v>
       </c>
       <c r="F631" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G631" s="2">
         <v>45921</v>
@@ -15949,22 +15937,22 @@
     </row>
     <row r="632" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A632" t="s">
-        <v>89</v>
+        <v>136</v>
       </c>
       <c r="B632">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C632" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="D632" t="s">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="E632">
-        <v>480</v>
+        <v>100</v>
       </c>
       <c r="F632" t="s">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="G632" s="2">
         <v>45921</v>
@@ -15972,19 +15960,19 @@
     </row>
     <row r="633" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A633" t="s">
-        <v>89</v>
+        <v>136</v>
       </c>
       <c r="B633">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C633" t="s">
-        <v>64</v>
+        <v>134</v>
       </c>
       <c r="D633" t="s">
-        <v>65</v>
+        <v>138</v>
       </c>
       <c r="E633">
-        <v>150</v>
+        <v>48</v>
       </c>
       <c r="F633" t="s">
         <v>10</v>
@@ -15995,22 +15983,22 @@
     </row>
     <row r="634" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A634" t="s">
-        <v>89</v>
+        <v>136</v>
       </c>
       <c r="B634">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C634" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D634" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E634">
-        <v>135</v>
+        <v>200</v>
       </c>
       <c r="F634" t="s">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="G634" s="2">
         <v>45921</v>
@@ -16021,19 +16009,19 @@
         <v>136</v>
       </c>
       <c r="B635">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C635" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D635" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E635">
-        <v>1</v>
+        <v>300</v>
       </c>
       <c r="F635" t="s">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="G635" s="2">
         <v>45921</v>
@@ -16041,22 +16029,22 @@
     </row>
     <row r="636" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A636" t="s">
-        <v>136</v>
+        <v>89</v>
       </c>
       <c r="B636">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C636" t="s">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="D636" t="s">
-        <v>48</v>
+        <v>91</v>
       </c>
       <c r="E636">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="F636" t="s">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="G636" s="2">
         <v>45921</v>
@@ -16064,19 +16052,19 @@
     </row>
     <row r="637" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A637" t="s">
-        <v>136</v>
+        <v>89</v>
       </c>
       <c r="B637">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C637" t="s">
-        <v>134</v>
+        <v>92</v>
       </c>
       <c r="D637" t="s">
-        <v>138</v>
+        <v>93</v>
       </c>
       <c r="E637">
-        <v>24</v>
+        <v>480</v>
       </c>
       <c r="F637" t="s">
         <v>10</v>
@@ -16087,10 +16075,10 @@
     </row>
     <row r="638" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A638" t="s">
-        <v>136</v>
+        <v>89</v>
       </c>
       <c r="B638">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C638" t="s">
         <v>64</v>
@@ -16099,10 +16087,10 @@
         <v>65</v>
       </c>
       <c r="E638">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F638" t="s">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="G638" s="2">
         <v>45921</v>
@@ -16110,22 +16098,22 @@
     </row>
     <row r="639" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A639" t="s">
-        <v>136</v>
+        <v>89</v>
       </c>
       <c r="B639">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C639" t="s">
+        <v>68</v>
+      </c>
+      <c r="D639" t="s">
+        <v>69</v>
+      </c>
+      <c r="E639">
         <v>135</v>
       </c>
-      <c r="D639" t="s">
-        <v>139</v>
-      </c>
-      <c r="E639">
-        <v>150</v>
-      </c>
       <c r="F639" t="s">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="G639" s="2">
         <v>45921</v>
@@ -16133,16 +16121,16 @@
     </row>
     <row r="640" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A640" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B640">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C640" t="s">
-        <v>181</v>
+        <v>58</v>
       </c>
       <c r="D640" t="s">
-        <v>182</v>
+        <v>59</v>
       </c>
       <c r="E640">
         <v>2</v>
@@ -16156,19 +16144,19 @@
     </row>
     <row r="641" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A641" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B641">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C641" t="s">
-        <v>96</v>
+        <v>60</v>
       </c>
       <c r="D641" t="s">
-        <v>190</v>
+        <v>61</v>
       </c>
       <c r="E641">
-        <v>200</v>
+        <v>468</v>
       </c>
       <c r="F641" t="s">
         <v>10</v>
@@ -16179,22 +16167,22 @@
     </row>
     <row r="642" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A642" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B642">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C642" t="s">
-        <v>110</v>
+        <v>62</v>
       </c>
       <c r="D642" t="s">
-        <v>117</v>
+        <v>63</v>
       </c>
       <c r="E642">
-        <v>0.2</v>
+        <v>300</v>
       </c>
       <c r="F642" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G642" s="2">
         <v>45921</v>
@@ -16202,19 +16190,19 @@
     </row>
     <row r="643" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A643" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B643">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C643" t="s">
-        <v>189</v>
+        <v>64</v>
       </c>
       <c r="D643" t="s">
-        <v>191</v>
+        <v>65</v>
       </c>
       <c r="E643">
-        <v>20</v>
+        <v>180</v>
       </c>
       <c r="F643" t="s">
         <v>10</v>
@@ -16225,22 +16213,22 @@
     </row>
     <row r="644" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A644" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B644">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C644" t="s">
-        <v>95</v>
+        <v>53</v>
       </c>
       <c r="D644" t="s">
-        <v>129</v>
+        <v>54</v>
       </c>
       <c r="E644">
-        <v>100</v>
+        <v>9.6000000000000014</v>
       </c>
       <c r="F644" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G644" s="2">
         <v>45921</v>
@@ -16248,22 +16236,22 @@
     </row>
     <row r="645" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A645" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B645">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C645" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D645" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E645">
-        <v>2</v>
+        <v>300</v>
       </c>
       <c r="F645" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G645" s="2">
         <v>45921</v>
@@ -16271,19 +16259,19 @@
     </row>
     <row r="646" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A646" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B646">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C646" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D646" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E646">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="F646" t="s">
         <v>10</v>
@@ -16294,19 +16282,19 @@
     </row>
     <row r="647" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A647" t="s">
-        <v>71</v>
+        <v>187</v>
       </c>
       <c r="B647">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C647" t="s">
-        <v>72</v>
+        <v>8</v>
       </c>
       <c r="D647" t="s">
-        <v>73</v>
+        <v>9</v>
       </c>
       <c r="E647">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="F647" t="s">
         <v>10</v>
@@ -16323,13 +16311,13 @@
         <v>4</v>
       </c>
       <c r="C648" t="s">
-        <v>28</v>
+        <v>72</v>
       </c>
       <c r="D648" t="s">
-        <v>29</v>
+        <v>73</v>
       </c>
       <c r="E648">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="F648" t="s">
         <v>10</v>
@@ -16346,10 +16334,10 @@
         <v>4</v>
       </c>
       <c r="C649" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="D649" t="s">
-        <v>75</v>
+        <v>29</v>
       </c>
       <c r="E649">
         <v>400</v>
@@ -16369,13 +16357,13 @@
         <v>4</v>
       </c>
       <c r="C650" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D650" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E650">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="F650" t="s">
         <v>10</v>
@@ -16392,16 +16380,16 @@
         <v>4</v>
       </c>
       <c r="C651" t="s">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="D651" t="s">
-        <v>19</v>
+        <v>77</v>
       </c>
       <c r="E651">
-        <v>16</v>
+        <v>200</v>
       </c>
       <c r="F651" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G651" s="2">
         <v>45921</v>
@@ -16415,16 +16403,16 @@
         <v>4</v>
       </c>
       <c r="C652" t="s">
-        <v>78</v>
+        <v>18</v>
       </c>
       <c r="D652" t="s">
-        <v>79</v>
+        <v>19</v>
       </c>
       <c r="E652">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F652" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G652" s="2">
         <v>45921</v>
@@ -16432,187 +16420,47 @@
     </row>
     <row r="653" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A653" t="s">
-        <v>187</v>
+        <v>71</v>
       </c>
       <c r="B653">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C653" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="D653" t="s">
-        <v>59</v>
+        <v>79</v>
       </c>
       <c r="E653">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F653" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G653" s="2">
         <v>45921</v>
       </c>
     </row>
     <row r="654" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A654" t="s">
-        <v>187</v>
-      </c>
-      <c r="B654">
-        <v>12</v>
-      </c>
-      <c r="C654" t="s">
-        <v>60</v>
-      </c>
-      <c r="D654" t="s">
-        <v>61</v>
-      </c>
-      <c r="E654">
-        <v>468</v>
-      </c>
-      <c r="F654" t="s">
-        <v>10</v>
-      </c>
-      <c r="G654" s="2">
-        <v>45921</v>
-      </c>
+      <c r="G654" s="2"/>
     </row>
     <row r="655" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A655" t="s">
-        <v>187</v>
-      </c>
-      <c r="B655">
-        <v>12</v>
-      </c>
-      <c r="C655" t="s">
-        <v>62</v>
-      </c>
-      <c r="D655" t="s">
-        <v>63</v>
-      </c>
-      <c r="E655">
-        <v>300</v>
-      </c>
-      <c r="F655" t="s">
-        <v>10</v>
-      </c>
-      <c r="G655" s="2">
-        <v>45921</v>
-      </c>
+      <c r="G655" s="2"/>
     </row>
     <row r="656" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A656" t="s">
-        <v>187</v>
-      </c>
-      <c r="B656">
-        <v>12</v>
-      </c>
-      <c r="C656" t="s">
-        <v>64</v>
-      </c>
-      <c r="D656" t="s">
-        <v>65</v>
-      </c>
-      <c r="E656">
-        <v>180</v>
-      </c>
-      <c r="F656" t="s">
-        <v>10</v>
-      </c>
-      <c r="G656" s="2">
-        <v>45921</v>
-      </c>
-    </row>
-    <row r="657" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A657" t="s">
-        <v>187</v>
-      </c>
-      <c r="B657">
-        <v>12</v>
-      </c>
-      <c r="C657" t="s">
-        <v>53</v>
-      </c>
-      <c r="D657" t="s">
-        <v>54</v>
-      </c>
-      <c r="E657">
-        <v>9.6</v>
-      </c>
-      <c r="F657" t="s">
-        <v>15</v>
-      </c>
-      <c r="G657" s="2">
-        <v>45921</v>
-      </c>
-    </row>
-    <row r="658" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A658" t="s">
-        <v>187</v>
-      </c>
-      <c r="B658">
-        <v>12</v>
-      </c>
-      <c r="C658" t="s">
-        <v>35</v>
-      </c>
-      <c r="D658" t="s">
-        <v>36</v>
-      </c>
-      <c r="E658">
-        <v>300</v>
-      </c>
-      <c r="F658" t="s">
-        <v>10</v>
-      </c>
-      <c r="G658" s="2">
-        <v>45921</v>
-      </c>
-    </row>
-    <row r="659" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A659" t="s">
-        <v>187</v>
-      </c>
-      <c r="B659">
-        <v>12</v>
-      </c>
-      <c r="C659" t="s">
-        <v>66</v>
-      </c>
-      <c r="D659" t="s">
-        <v>67</v>
-      </c>
-      <c r="E659">
-        <v>180</v>
-      </c>
-      <c r="F659" t="s">
-        <v>10</v>
-      </c>
-      <c r="G659" s="2">
-        <v>45921</v>
-      </c>
-    </row>
-    <row r="660" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A660" t="s">
-        <v>187</v>
-      </c>
-      <c r="B660">
-        <v>12</v>
-      </c>
-      <c r="C660" t="s">
-        <v>8</v>
-      </c>
-      <c r="D660" t="s">
-        <v>9</v>
-      </c>
-      <c r="E660">
-        <v>1200</v>
-      </c>
-      <c r="F660" t="s">
-        <v>10</v>
-      </c>
-      <c r="G660" s="2">
-        <v>45921</v>
-      </c>
+      <c r="G656" s="2"/>
+    </row>
+    <row r="657" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G657" s="2"/>
+    </row>
+    <row r="658" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G658" s="2"/>
+    </row>
+    <row r="659" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G659" s="2"/>
+    </row>
+    <row r="660" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G660" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -16629,7 +16477,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D666"/>
+  <dimension ref="A1:D676"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -25654,10 +25502,10 @@
     </row>
     <row r="645" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A645" t="s">
-        <v>188</v>
+        <v>101</v>
       </c>
       <c r="B645">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C645" t="s">
         <v>15</v>
@@ -25668,10 +25516,10 @@
     </row>
     <row r="646" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A646" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B646">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C646" t="s">
         <v>15</v>
@@ -25682,10 +25530,10 @@
     </row>
     <row r="647" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A647" t="s">
-        <v>102</v>
+        <v>133</v>
       </c>
       <c r="B647">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C647" t="s">
         <v>15</v>
@@ -25699,7 +25547,7 @@
         <v>94</v>
       </c>
       <c r="B648">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C648" t="s">
         <v>15</v>
@@ -25724,10 +25572,10 @@
     </row>
     <row r="650" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A650" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="B650">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="C650" t="s">
         <v>10</v>
@@ -25738,13 +25586,13 @@
     </row>
     <row r="651" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A651" t="s">
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="B651">
-        <v>2</v>
+        <v>300</v>
       </c>
       <c r="C651" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D651" s="2">
         <v>45921</v>
@@ -25752,13 +25600,13 @@
     </row>
     <row r="652" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A652" t="s">
-        <v>43</v>
+        <v>95</v>
       </c>
       <c r="B652">
-        <v>750</v>
+        <v>2</v>
       </c>
       <c r="C652" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D652" s="2">
         <v>45921</v>
@@ -25766,13 +25614,13 @@
     </row>
     <row r="653" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A653" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="B653">
-        <v>35</v>
+        <v>750</v>
       </c>
       <c r="C653" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D653" s="2">
         <v>45921</v>
@@ -25780,10 +25628,10 @@
     </row>
     <row r="654" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A654" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B654">
-        <v>1</v>
+        <v>44.6</v>
       </c>
       <c r="C654" t="s">
         <v>15</v>
@@ -25794,13 +25642,13 @@
     </row>
     <row r="655" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A655" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="B655">
-        <v>1</v>
+        <v>400</v>
       </c>
       <c r="C655" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D655" s="2">
         <v>45921</v>
@@ -25808,10 +25656,10 @@
     </row>
     <row r="656" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A656" t="s">
-        <v>142</v>
+        <v>178</v>
       </c>
       <c r="B656">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C656" t="s">
         <v>15</v>
@@ -25822,10 +25670,10 @@
     </row>
     <row r="657" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A657" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="B657">
-        <v>135</v>
+        <v>8</v>
       </c>
       <c r="C657" t="s">
         <v>10</v>
@@ -25836,13 +25684,13 @@
     </row>
     <row r="658" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A658" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="B658">
-        <v>3</v>
+        <v>1000</v>
       </c>
       <c r="C658" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D658" s="2">
         <v>45921</v>
@@ -25850,13 +25698,13 @@
     </row>
     <row r="659" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A659" t="s">
-        <v>109</v>
+        <v>47</v>
       </c>
       <c r="B659">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="C659" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D659" s="2">
         <v>45921</v>
@@ -25864,10 +25712,10 @@
     </row>
     <row r="660" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A660" t="s">
-        <v>92</v>
+        <v>18</v>
       </c>
       <c r="B660">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C660" t="s">
         <v>15</v>
@@ -25878,13 +25726,13 @@
     </row>
     <row r="661" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A661" t="s">
-        <v>135</v>
+        <v>66</v>
       </c>
       <c r="B661">
-        <v>1</v>
+        <v>180</v>
       </c>
       <c r="C661" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D661" s="2">
         <v>45921</v>
@@ -25892,10 +25740,10 @@
     </row>
     <row r="662" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A662" t="s">
-        <v>8</v>
+        <v>134</v>
       </c>
       <c r="B662">
-        <v>1200</v>
+        <v>48</v>
       </c>
       <c r="C662" t="s">
         <v>10</v>
@@ -25906,10 +25754,10 @@
     </row>
     <row r="663" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A663" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B663">
-        <v>250</v>
+        <v>530</v>
       </c>
       <c r="C663" t="s">
         <v>10</v>
@@ -25920,10 +25768,10 @@
     </row>
     <row r="664" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A664" t="s">
-        <v>110</v>
+        <v>188</v>
       </c>
       <c r="B664">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="C664" t="s">
         <v>15</v>
@@ -25934,13 +25782,13 @@
     </row>
     <row r="665" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A665" t="s">
-        <v>189</v>
+        <v>60</v>
       </c>
       <c r="B665">
-        <v>1</v>
+        <v>468</v>
       </c>
       <c r="C665" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D665" s="2">
         <v>45921</v>
@@ -25948,17 +25796,146 @@
     </row>
     <row r="666" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A666" t="s">
-        <v>193</v>
+        <v>74</v>
       </c>
       <c r="B666">
-        <v>1</v>
+        <v>400</v>
       </c>
       <c r="C666" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D666" s="2">
         <v>45921</v>
       </c>
+    </row>
+    <row r="667" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A667" t="s">
+        <v>68</v>
+      </c>
+      <c r="B667">
+        <v>135</v>
+      </c>
+      <c r="C667" t="s">
+        <v>10</v>
+      </c>
+      <c r="D667" s="2">
+        <v>45921</v>
+      </c>
+    </row>
+    <row r="668" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A668" t="s">
+        <v>96</v>
+      </c>
+      <c r="B668">
+        <v>3</v>
+      </c>
+      <c r="C668" t="s">
+        <v>15</v>
+      </c>
+      <c r="D668" s="2">
+        <v>45921</v>
+      </c>
+    </row>
+    <row r="669" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A669" t="s">
+        <v>109</v>
+      </c>
+      <c r="B669">
+        <v>1</v>
+      </c>
+      <c r="C669" t="s">
+        <v>15</v>
+      </c>
+      <c r="D669" s="2">
+        <v>45921</v>
+      </c>
+    </row>
+    <row r="670" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A670" t="s">
+        <v>90</v>
+      </c>
+      <c r="B670">
+        <v>300</v>
+      </c>
+      <c r="C670" t="s">
+        <v>10</v>
+      </c>
+      <c r="D670" s="2">
+        <v>45921</v>
+      </c>
+    </row>
+    <row r="671" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A671" t="s">
+        <v>92</v>
+      </c>
+      <c r="B671">
+        <v>480</v>
+      </c>
+      <c r="C671" t="s">
+        <v>10</v>
+      </c>
+      <c r="D671" s="2">
+        <v>45921</v>
+      </c>
+    </row>
+    <row r="672" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A672" t="s">
+        <v>135</v>
+      </c>
+      <c r="B672">
+        <v>300</v>
+      </c>
+      <c r="C672" t="s">
+        <v>10</v>
+      </c>
+      <c r="D672" s="2">
+        <v>45921</v>
+      </c>
+    </row>
+    <row r="673" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A673" t="s">
+        <v>8</v>
+      </c>
+      <c r="B673">
+        <v>1200</v>
+      </c>
+      <c r="C673" t="s">
+        <v>10</v>
+      </c>
+      <c r="D673" s="2">
+        <v>45921</v>
+      </c>
+    </row>
+    <row r="674" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A674" t="s">
+        <v>62</v>
+      </c>
+      <c r="B674">
+        <v>300</v>
+      </c>
+      <c r="C674" t="s">
+        <v>10</v>
+      </c>
+      <c r="D674" s="2">
+        <v>45921</v>
+      </c>
+    </row>
+    <row r="675" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A675" t="s">
+        <v>189</v>
+      </c>
+      <c r="B675">
+        <v>1</v>
+      </c>
+      <c r="C675" t="s">
+        <v>15</v>
+      </c>
+      <c r="D675" s="2">
+        <v>45921</v>
+      </c>
+    </row>
+    <row r="676" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D676" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>